<commit_message>
Corregido mapeo de marcaciones biometricas H.E. (Inicio de horas extra / Fin de horas extra). Ahora se leen e identifican correctamente las marcaciones biometricas de Raul Espinoza a las 19:48 y 23:48
</commit_message>
<xml_diff>
--- a/Sistema_Asistencia_GZG_v1.0.xlsx
+++ b/Sistema_Asistencia_GZG_v1.0.xlsx
@@ -2073,12 +2073,12 @@
       </c>
       <c r="M17" s="6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="N17" s="6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>18:17</t>
         </is>
       </c>
       <c r="O17" s="6" t="inlineStr">
@@ -2529,22 +2529,22 @@
       </c>
       <c r="M21" s="6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="N21" s="6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>19:48</t>
         </is>
       </c>
       <c r="O21" s="6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="P21" s="6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>23:48</t>
         </is>
       </c>
       <c r="Q21" s="6" t="inlineStr">
@@ -2564,7 +2564,7 @@
       </c>
       <c r="T21" s="6" t="inlineStr">
         <is>
-          <t>00:23</t>
+          <t>04:23</t>
         </is>
       </c>
       <c r="U21" s="6" t="inlineStr">
@@ -5031,12 +5031,12 @@
       </c>
       <c r="M43" s="6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="N43" s="6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>18:56</t>
         </is>
       </c>
       <c r="O43" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Eliminado fallback de HE. Estado Indefinido se ignora por completo. Inicio/Fin H.E. solo provienen estrictamente de marcaciones explicitas Inicio de horas extra y Fin de horas extra
</commit_message>
<xml_diff>
--- a/Sistema_Asistencia_GZG_v1.0.xlsx
+++ b/Sistema_Asistencia_GZG_v1.0.xlsx
@@ -2073,12 +2073,12 @@
       </c>
       <c r="M17" s="6" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N17" s="6" t="inlineStr">
         <is>
-          <t>18:17</t>
+          <t>-</t>
         </is>
       </c>
       <c r="O17" s="6" t="inlineStr">
@@ -2529,22 +2529,22 @@
       </c>
       <c r="M21" s="6" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N21" s="6" t="inlineStr">
         <is>
-          <t>19:48</t>
+          <t>-</t>
         </is>
       </c>
       <c r="O21" s="6" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>-</t>
         </is>
       </c>
       <c r="P21" s="6" t="inlineStr">
         <is>
-          <t>23:48</t>
+          <t>-</t>
         </is>
       </c>
       <c r="Q21" s="6" t="inlineStr">
@@ -2564,7 +2564,7 @@
       </c>
       <c r="T21" s="6" t="inlineStr">
         <is>
-          <t>04:23</t>
+          <t>00:23</t>
         </is>
       </c>
       <c r="U21" s="6" t="inlineStr">
@@ -5031,12 +5031,12 @@
       </c>
       <c r="M43" s="6" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N43" s="6" t="inlineStr">
         <is>
-          <t>18:56</t>
+          <t>-</t>
         </is>
       </c>
       <c r="O43" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Solucionado matcheo flexible de DNIs omitiendo ceros a la izquierda (lstrip). Ahora los DNIs como 03208053 (Franco Moreto Bermeo) y 006616501 (Yenkli Vicente Ordoñez Arteaga) se reconocen al 100% y se exportan con su DNI oficial sin marcar DESCONOCIDO
</commit_message>
<xml_diff>
--- a/Sistema_Asistencia_GZG_v1.0.xlsx
+++ b/Sistema_Asistencia_GZG_v1.0.xlsx
@@ -486,7 +486,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W115"/>
+  <dimension ref="A1:W112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -649,17 +649,17 @@
     <row r="5" ht="20" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>18074244</t>
+          <t>006616501</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>LAZARO CRUZ</t>
+          <t>ORDOÑEZ ARTEAGA</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>RAUL RICHARD</t>
+          <t>YENKLI VICENTE</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
@@ -669,7 +669,7 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>MAQUINARIA PESADA</t>
+          <t>ELECTRICIDAD</t>
         </is>
       </c>
       <c r="F5" s="6" t="inlineStr">
@@ -694,7 +694,7 @@
       </c>
       <c r="J5" s="6" t="inlineStr">
         <is>
-          <t>07:04</t>
+          <t>06:49</t>
         </is>
       </c>
       <c r="K5" s="6" t="inlineStr">
@@ -704,7 +704,7 @@
       </c>
       <c r="L5" s="6" t="inlineStr">
         <is>
-          <t>19:19</t>
+          <t>20:17</t>
         </is>
       </c>
       <c r="M5" s="6" t="inlineStr">
@@ -729,7 +729,7 @@
       </c>
       <c r="Q5" s="6" t="inlineStr">
         <is>
-          <t>12:15</t>
+          <t>13:28</t>
         </is>
       </c>
       <c r="R5" s="6" t="inlineStr">
@@ -739,40 +739,44 @@
       </c>
       <c r="S5" s="6" t="inlineStr">
         <is>
-          <t>00:19</t>
+          <t>01:17</t>
         </is>
       </c>
       <c r="T5" s="6" t="inlineStr">
         <is>
-          <t>00:19</t>
+          <t>01:17</t>
         </is>
       </c>
       <c r="U5" s="6" t="inlineStr">
         <is>
-          <t>Imagen de cara</t>
+          <t>-</t>
         </is>
       </c>
       <c r="V5" s="6" t="inlineStr">
         <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="W5" s="5" t="inlineStr"/>
+          <t>Duplicado (Entrada)</t>
+        </is>
+      </c>
+      <c r="W5" s="5" t="inlineStr">
+        <is>
+          <t>Entrada duplicada (20:15), Exceso de jornada no autorizado (77 min)</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>18074244</t>
+          <t>006616501</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>LAZARO CRUZ</t>
+          <t>ORDOÑEZ ARTEAGA</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>RAUL RICHARD</t>
+          <t>YENKLI VICENTE</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
@@ -782,7 +786,7 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>MAQUINARIA PESADA</t>
+          <t>ELECTRICIDAD</t>
         </is>
       </c>
       <c r="F6" s="6" t="inlineStr">
@@ -807,7 +811,7 @@
       </c>
       <c r="J6" s="6" t="inlineStr">
         <is>
-          <t>06:30</t>
+          <t>06:41</t>
         </is>
       </c>
       <c r="K6" s="6" t="inlineStr">
@@ -817,7 +821,7 @@
       </c>
       <c r="L6" s="6" t="inlineStr">
         <is>
-          <t>18:57</t>
+          <t>21:37</t>
         </is>
       </c>
       <c r="M6" s="6" t="inlineStr">
@@ -842,7 +846,7 @@
       </c>
       <c r="Q6" s="6" t="inlineStr">
         <is>
-          <t>12:27</t>
+          <t>14:56</t>
         </is>
       </c>
       <c r="R6" s="6" t="inlineStr">
@@ -852,17 +856,17 @@
       </c>
       <c r="S6" s="6" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>02:37</t>
         </is>
       </c>
       <c r="T6" s="6" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>02:37</t>
         </is>
       </c>
       <c r="U6" s="6" t="inlineStr">
         <is>
-          <t>Huella dactilar</t>
+          <t>Imagen de cara</t>
         </is>
       </c>
       <c r="V6" s="6" t="inlineStr">
@@ -870,22 +874,26 @@
           <t>Normal</t>
         </is>
       </c>
-      <c r="W6" s="5" t="inlineStr"/>
+      <c r="W6" s="5" t="inlineStr">
+        <is>
+          <t>Exceso de jornada no autorizado (157 min)</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="20" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>18861684</t>
+          <t>03208053</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>ZAMORA CARRASCO</t>
+          <t>MORETO BERMEO</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>JACOB</t>
+          <t>FRANCO</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
@@ -895,17 +903,17 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>ELECTRICIDAD</t>
+          <t>MANTENIMIENTO</t>
         </is>
       </c>
       <c r="F7" s="6" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="G7" s="6" t="inlineStr">
         <is>
-          <t>Lunes</t>
+          <t>Martes</t>
         </is>
       </c>
       <c r="H7" s="6" t="inlineStr">
@@ -915,22 +923,22 @@
       </c>
       <c r="I7" s="6" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="J7" s="6" t="inlineStr">
         <is>
-          <t>06:48</t>
+          <t>06:30</t>
         </is>
       </c>
       <c r="K7" s="6" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="L7" s="6" t="inlineStr">
         <is>
-          <t>19:10</t>
+          <t>18:55</t>
         </is>
       </c>
       <c r="M7" s="6" t="inlineStr">
@@ -955,7 +963,7 @@
       </c>
       <c r="Q7" s="6" t="inlineStr">
         <is>
-          <t>12:22</t>
+          <t>12:25</t>
         </is>
       </c>
       <c r="R7" s="6" t="inlineStr">
@@ -965,12 +973,12 @@
       </c>
       <c r="S7" s="6" t="inlineStr">
         <is>
-          <t>00:10</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="T7" s="6" t="inlineStr">
         <is>
-          <t>00:10</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="U7" s="6" t="inlineStr">
@@ -988,17 +996,17 @@
     <row r="8" ht="20" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>18861684</t>
+          <t>18074244</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>ZAMORA CARRASCO</t>
+          <t>LAZARO CRUZ</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>JACOB</t>
+          <t>RAUL RICHARD</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
@@ -1008,17 +1016,17 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>ELECTRICIDAD</t>
+          <t>MAQUINARIA PESADA</t>
         </is>
       </c>
       <c r="F8" s="6" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="G8" s="6" t="inlineStr">
         <is>
-          <t>Martes</t>
+          <t>Lunes</t>
         </is>
       </c>
       <c r="H8" s="6" t="inlineStr">
@@ -1028,22 +1036,22 @@
       </c>
       <c r="I8" s="6" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="J8" s="6" t="inlineStr">
         <is>
-          <t>06:44</t>
+          <t>07:04</t>
         </is>
       </c>
       <c r="K8" s="6" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="L8" s="6" t="inlineStr">
         <is>
-          <t>19:14</t>
+          <t>19:19</t>
         </is>
       </c>
       <c r="M8" s="6" t="inlineStr">
@@ -1068,7 +1076,7 @@
       </c>
       <c r="Q8" s="6" t="inlineStr">
         <is>
-          <t>12:30</t>
+          <t>12:15</t>
         </is>
       </c>
       <c r="R8" s="6" t="inlineStr">
@@ -1078,17 +1086,17 @@
       </c>
       <c r="S8" s="6" t="inlineStr">
         <is>
-          <t>00:14</t>
+          <t>00:19</t>
         </is>
       </c>
       <c r="T8" s="6" t="inlineStr">
         <is>
-          <t>00:14</t>
+          <t>00:19</t>
         </is>
       </c>
       <c r="U8" s="6" t="inlineStr">
         <is>
-          <t>Huella dactilar</t>
+          <t>Imagen de cara</t>
         </is>
       </c>
       <c r="V8" s="6" t="inlineStr">
@@ -1101,23 +1109,27 @@
     <row r="9" ht="20" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>3208053</t>
+          <t>18074244</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>DESCONOCIDO</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="inlineStr"/>
+          <t>LAZARO CRUZ</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>RAUL RICHARD</t>
+        </is>
+      </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>OPER&amp;MTTO</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>MAQUINARIA PESADA</t>
         </is>
       </c>
       <c r="F9" s="6" t="inlineStr">
@@ -1152,7 +1164,7 @@
       </c>
       <c r="L9" s="6" t="inlineStr">
         <is>
-          <t>18:55</t>
+          <t>18:57</t>
         </is>
       </c>
       <c r="M9" s="6" t="inlineStr">
@@ -1177,7 +1189,7 @@
       </c>
       <c r="Q9" s="6" t="inlineStr">
         <is>
-          <t>12:25</t>
+          <t>12:27</t>
         </is>
       </c>
       <c r="R9" s="6" t="inlineStr">
@@ -1210,17 +1222,17 @@
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>40829439</t>
+          <t>18861684</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>CASTRO ESCOBEDO</t>
+          <t>ZAMORA CARRASCO</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>RONALD SLIM</t>
+          <t>JACOB</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
@@ -1230,7 +1242,7 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>MAESTRANZA</t>
+          <t>ELECTRICIDAD</t>
         </is>
       </c>
       <c r="F10" s="6" t="inlineStr">
@@ -1255,7 +1267,7 @@
       </c>
       <c r="J10" s="6" t="inlineStr">
         <is>
-          <t>06:47</t>
+          <t>06:48</t>
         </is>
       </c>
       <c r="K10" s="6" t="inlineStr">
@@ -1265,7 +1277,7 @@
       </c>
       <c r="L10" s="6" t="inlineStr">
         <is>
-          <t>20:56</t>
+          <t>19:10</t>
         </is>
       </c>
       <c r="M10" s="6" t="inlineStr">
@@ -1290,7 +1302,7 @@
       </c>
       <c r="Q10" s="6" t="inlineStr">
         <is>
-          <t>14:09</t>
+          <t>12:22</t>
         </is>
       </c>
       <c r="R10" s="6" t="inlineStr">
@@ -1300,12 +1312,12 @@
       </c>
       <c r="S10" s="6" t="inlineStr">
         <is>
-          <t>01:56</t>
+          <t>00:10</t>
         </is>
       </c>
       <c r="T10" s="6" t="inlineStr">
         <is>
-          <t>01:56</t>
+          <t>00:10</t>
         </is>
       </c>
       <c r="U10" s="6" t="inlineStr">
@@ -1318,26 +1330,22 @@
           <t>Normal</t>
         </is>
       </c>
-      <c r="W10" s="5" t="inlineStr">
-        <is>
-          <t>Exceso de jornada no autorizado (116 min)</t>
-        </is>
-      </c>
+      <c r="W10" s="5" t="inlineStr"/>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>40829439</t>
+          <t>18861684</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>CASTRO ESCOBEDO</t>
+          <t>ZAMORA CARRASCO</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>RONALD SLIM</t>
+          <t>JACOB</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
@@ -1347,7 +1355,7 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>MAESTRANZA</t>
+          <t>ELECTRICIDAD</t>
         </is>
       </c>
       <c r="F11" s="6" t="inlineStr">
@@ -1372,7 +1380,7 @@
       </c>
       <c r="J11" s="6" t="inlineStr">
         <is>
-          <t>06:43</t>
+          <t>06:44</t>
         </is>
       </c>
       <c r="K11" s="6" t="inlineStr">
@@ -1407,7 +1415,7 @@
       </c>
       <c r="Q11" s="6" t="inlineStr">
         <is>
-          <t>12:31</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="R11" s="6" t="inlineStr">
@@ -1440,17 +1448,17 @@
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>41219221</t>
+          <t>40829439</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>VIGO RAFAEL</t>
+          <t>CASTRO ESCOBEDO</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>JOSE ISMAEL</t>
+          <t>RONALD SLIM</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
@@ -1460,7 +1468,7 @@
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>MANTENIMIENTO</t>
+          <t>MAESTRANZA</t>
         </is>
       </c>
       <c r="F12" s="6" t="inlineStr">
@@ -1485,11 +1493,19 @@
       </c>
       <c r="J12" s="6" t="inlineStr">
         <is>
-          <t>06:46</t>
-        </is>
-      </c>
-      <c r="K12" s="6" t="inlineStr"/>
-      <c r="L12" s="6" t="inlineStr"/>
+          <t>06:47</t>
+        </is>
+      </c>
+      <c r="K12" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="L12" s="6" t="inlineStr">
+        <is>
+          <t>20:56</t>
+        </is>
+      </c>
       <c r="M12" s="6" t="inlineStr">
         <is>
           <t>-</t>
@@ -1512,7 +1528,7 @@
       </c>
       <c r="Q12" s="6" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>14:09</t>
         </is>
       </c>
       <c r="R12" s="6" t="inlineStr">
@@ -1522,17 +1538,17 @@
       </c>
       <c r="S12" s="6" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>01:56</t>
         </is>
       </c>
       <c r="T12" s="6" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>01:56</t>
         </is>
       </c>
       <c r="U12" s="6" t="inlineStr">
         <is>
-          <t>Imagen de cara</t>
+          <t>Huella dactilar</t>
         </is>
       </c>
       <c r="V12" s="6" t="inlineStr">
@@ -1542,24 +1558,24 @@
       </c>
       <c r="W12" s="5" t="inlineStr">
         <is>
-          <t>Falta marcación de salida</t>
+          <t>Exceso de jornada no autorizado (116 min)</t>
         </is>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>41219221</t>
+          <t>40829439</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>VIGO RAFAEL</t>
+          <t>CASTRO ESCOBEDO</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>JOSE ISMAEL</t>
+          <t>RONALD SLIM</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
@@ -1569,7 +1585,7 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>MANTENIMIENTO</t>
+          <t>MAESTRANZA</t>
         </is>
       </c>
       <c r="F13" s="6" t="inlineStr">
@@ -1594,7 +1610,7 @@
       </c>
       <c r="J13" s="6" t="inlineStr">
         <is>
-          <t>06:37</t>
+          <t>06:43</t>
         </is>
       </c>
       <c r="K13" s="6" t="inlineStr">
@@ -1604,7 +1620,7 @@
       </c>
       <c r="L13" s="6" t="inlineStr">
         <is>
-          <t>18:50</t>
+          <t>19:14</t>
         </is>
       </c>
       <c r="M13" s="6" t="inlineStr">
@@ -1629,7 +1645,7 @@
       </c>
       <c r="Q13" s="6" t="inlineStr">
         <is>
-          <t>12:13</t>
+          <t>12:31</t>
         </is>
       </c>
       <c r="R13" s="6" t="inlineStr">
@@ -1639,12 +1655,12 @@
       </c>
       <c r="S13" s="6" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>00:14</t>
         </is>
       </c>
       <c r="T13" s="6" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>00:14</t>
         </is>
       </c>
       <c r="U13" s="6" t="inlineStr">
@@ -1662,17 +1678,17 @@
     <row r="14" ht="20" customHeight="1">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>42300003</t>
+          <t>41219221</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>CELEN RUIZ</t>
+          <t>VIGO RAFAEL</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>ISAAC ENCARNACION</t>
+          <t>JOSE ISMAEL</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
@@ -1682,7 +1698,7 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>OPERACIONES</t>
+          <t>MANTENIMIENTO</t>
         </is>
       </c>
       <c r="F14" s="6" t="inlineStr">
@@ -1697,7 +1713,7 @@
       </c>
       <c r="H14" s="6" t="inlineStr">
         <is>
-          <t>NOCHE</t>
+          <t>DIA</t>
         </is>
       </c>
       <c r="I14" s="6" t="inlineStr">
@@ -1707,7 +1723,7 @@
       </c>
       <c r="J14" s="6" t="inlineStr">
         <is>
-          <t>18:16</t>
+          <t>06:46</t>
         </is>
       </c>
       <c r="K14" s="6" t="inlineStr"/>
@@ -1754,34 +1770,34 @@
       </c>
       <c r="U14" s="6" t="inlineStr">
         <is>
-          <t>Huella dactilar</t>
+          <t>Imagen de cara</t>
         </is>
       </c>
       <c r="V14" s="6" t="inlineStr">
         <is>
-          <t>Duplicado (Entrada)</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="W14" s="5" t="inlineStr">
         <is>
-          <t>Entrada duplicada (18:17)</t>
+          <t>Falta marcación de salida</t>
         </is>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>42300003</t>
+          <t>41219221</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>CELEN RUIZ</t>
+          <t>VIGO RAFAEL</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>ISAAC ENCARNACION</t>
+          <t>JOSE ISMAEL</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
@@ -1791,7 +1807,7 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>OPERACIONES</t>
+          <t>MANTENIMIENTO</t>
         </is>
       </c>
       <c r="F15" s="6" t="inlineStr">
@@ -1806,11 +1822,19 @@
       </c>
       <c r="H15" s="6" t="inlineStr">
         <is>
-          <t>NOCHE</t>
-        </is>
-      </c>
-      <c r="I15" s="6" t="inlineStr"/>
-      <c r="J15" s="6" t="inlineStr"/>
+          <t>DIA</t>
+        </is>
+      </c>
+      <c r="I15" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="J15" s="6" t="inlineStr">
+        <is>
+          <t>06:37</t>
+        </is>
+      </c>
       <c r="K15" s="6" t="inlineStr">
         <is>
           <t>2026-08-18</t>
@@ -1818,7 +1842,7 @@
       </c>
       <c r="L15" s="6" t="inlineStr">
         <is>
-          <t>07:01</t>
+          <t>18:50</t>
         </is>
       </c>
       <c r="M15" s="6" t="inlineStr">
@@ -1843,7 +1867,7 @@
       </c>
       <c r="Q15" s="6" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>12:13</t>
         </is>
       </c>
       <c r="R15" s="6" t="inlineStr">
@@ -1863,34 +1887,30 @@
       </c>
       <c r="U15" s="6" t="inlineStr">
         <is>
-          <t>Imagen de cara</t>
+          <t>Huella dactilar</t>
         </is>
       </c>
       <c r="V15" s="6" t="inlineStr">
         <is>
-          <t>Salida sin entrada</t>
-        </is>
-      </c>
-      <c r="W15" s="5" t="inlineStr">
-        <is>
-          <t>Salida sin registro de entrada previa (07:01)</t>
-        </is>
-      </c>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="W15" s="5" t="inlineStr"/>
     </row>
     <row r="16" ht="20" customHeight="1">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>42626422</t>
+          <t>42300003</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>ALVARADO BERMEO</t>
+          <t>CELEN RUIZ</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>NEPTALI</t>
+          <t>ISAAC ENCARNACION</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
@@ -1915,7 +1935,7 @@
       </c>
       <c r="H16" s="6" t="inlineStr">
         <is>
-          <t>DIA</t>
+          <t>NOCHE</t>
         </is>
       </c>
       <c r="I16" s="6" t="inlineStr">
@@ -1925,19 +1945,11 @@
       </c>
       <c r="J16" s="6" t="inlineStr">
         <is>
-          <t>06:39</t>
-        </is>
-      </c>
-      <c r="K16" s="6" t="inlineStr">
-        <is>
-          <t>2026-08-17</t>
-        </is>
-      </c>
-      <c r="L16" s="6" t="inlineStr">
-        <is>
-          <t>19:01</t>
-        </is>
-      </c>
+          <t>18:16</t>
+        </is>
+      </c>
+      <c r="K16" s="6" t="inlineStr"/>
+      <c r="L16" s="6" t="inlineStr"/>
       <c r="M16" s="6" t="inlineStr">
         <is>
           <t>-</t>
@@ -1960,7 +1972,7 @@
       </c>
       <c r="Q16" s="6" t="inlineStr">
         <is>
-          <t>12:22</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="R16" s="6" t="inlineStr">
@@ -1970,40 +1982,44 @@
       </c>
       <c r="S16" s="6" t="inlineStr">
         <is>
-          <t>00:01</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="T16" s="6" t="inlineStr">
         <is>
-          <t>00:01</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="U16" s="6" t="inlineStr">
         <is>
-          <t>Huella dactilar</t>
+          <t>-</t>
         </is>
       </c>
       <c r="V16" s="6" t="inlineStr">
         <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="W16" s="5" t="inlineStr"/>
+          <t>Duplicado (Entrada)</t>
+        </is>
+      </c>
+      <c r="W16" s="5" t="inlineStr">
+        <is>
+          <t>Entrada duplicada (18:17)</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="20" customHeight="1">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>42626422</t>
+          <t>42300003</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>ALVARADO BERMEO</t>
+          <t>CELEN RUIZ</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>NEPTALI</t>
+          <t>ISAAC ENCARNACION</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
@@ -2028,19 +2044,11 @@
       </c>
       <c r="H17" s="6" t="inlineStr">
         <is>
-          <t>DIA</t>
-        </is>
-      </c>
-      <c r="I17" s="6" t="inlineStr">
-        <is>
-          <t>2026-08-18</t>
-        </is>
-      </c>
-      <c r="J17" s="6" t="inlineStr">
-        <is>
-          <t>06:37</t>
-        </is>
-      </c>
+          <t>NOCHE</t>
+        </is>
+      </c>
+      <c r="I17" s="6" t="inlineStr"/>
+      <c r="J17" s="6" t="inlineStr"/>
       <c r="K17" s="6" t="inlineStr">
         <is>
           <t>2026-08-18</t>
@@ -2048,7 +2056,7 @@
       </c>
       <c r="L17" s="6" t="inlineStr">
         <is>
-          <t>19:02</t>
+          <t>07:01</t>
         </is>
       </c>
       <c r="M17" s="6" t="inlineStr">
@@ -2073,7 +2081,7 @@
       </c>
       <c r="Q17" s="6" t="inlineStr">
         <is>
-          <t>12:25</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="R17" s="6" t="inlineStr">
@@ -2083,40 +2091,44 @@
       </c>
       <c r="S17" s="6" t="inlineStr">
         <is>
-          <t>00:02</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="T17" s="6" t="inlineStr">
         <is>
-          <t>00:02</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="U17" s="6" t="inlineStr">
         <is>
-          <t>Huella dactilar</t>
+          <t>Imagen de cara</t>
         </is>
       </c>
       <c r="V17" s="6" t="inlineStr">
         <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="W17" s="5" t="inlineStr"/>
+          <t>Salida sin entrada</t>
+        </is>
+      </c>
+      <c r="W17" s="5" t="inlineStr">
+        <is>
+          <t>Salida sin registro de entrada previa (07:01)</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="20" customHeight="1">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>44196392</t>
+          <t>42626422</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>BERMEO SANTOS</t>
+          <t>ALVARADO BERMEO</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>ALEXANDER</t>
+          <t>NEPTALI</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
@@ -2126,17 +2138,17 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>MANTENIMIENTO</t>
+          <t>OPERACIONES</t>
         </is>
       </c>
       <c r="F18" s="6" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="G18" s="6" t="inlineStr">
         <is>
-          <t>Martes</t>
+          <t>Lunes</t>
         </is>
       </c>
       <c r="H18" s="6" t="inlineStr">
@@ -2146,22 +2158,22 @@
       </c>
       <c r="I18" s="6" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="J18" s="6" t="inlineStr">
         <is>
-          <t>06:35</t>
+          <t>06:39</t>
         </is>
       </c>
       <c r="K18" s="6" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="L18" s="6" t="inlineStr">
         <is>
-          <t>18:54</t>
+          <t>19:01</t>
         </is>
       </c>
       <c r="M18" s="6" t="inlineStr">
@@ -2186,7 +2198,7 @@
       </c>
       <c r="Q18" s="6" t="inlineStr">
         <is>
-          <t>12:19</t>
+          <t>12:22</t>
         </is>
       </c>
       <c r="R18" s="6" t="inlineStr">
@@ -2196,12 +2208,12 @@
       </c>
       <c r="S18" s="6" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>00:01</t>
         </is>
       </c>
       <c r="T18" s="6" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>00:01</t>
         </is>
       </c>
       <c r="U18" s="6" t="inlineStr">
@@ -2219,17 +2231,17 @@
     <row r="19" ht="20" customHeight="1">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>44955960</t>
+          <t>42626422</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>ESPINOZA SAAVEDRA</t>
+          <t>ALVARADO BERMEO</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>RAUL ESTEBAN</t>
+          <t>NEPTALI</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
@@ -2239,17 +2251,17 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>COMUNICACIONES</t>
+          <t>OPERACIONES</t>
         </is>
       </c>
       <c r="F19" s="6" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="G19" s="6" t="inlineStr">
         <is>
-          <t>Lunes</t>
+          <t>Martes</t>
         </is>
       </c>
       <c r="H19" s="6" t="inlineStr">
@@ -2259,47 +2271,47 @@
       </c>
       <c r="I19" s="6" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="J19" s="6" t="inlineStr">
         <is>
-          <t>06:49</t>
+          <t>06:37</t>
         </is>
       </c>
       <c r="K19" s="6" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="L19" s="6" t="inlineStr">
         <is>
-          <t>19:23</t>
+          <t>19:02</t>
         </is>
       </c>
       <c r="M19" s="6" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N19" s="6" t="inlineStr">
         <is>
-          <t>19:48</t>
+          <t>-</t>
         </is>
       </c>
       <c r="O19" s="6" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>-</t>
         </is>
       </c>
       <c r="P19" s="6" t="inlineStr">
         <is>
-          <t>23:48</t>
+          <t>-</t>
         </is>
       </c>
       <c r="Q19" s="6" t="inlineStr">
         <is>
-          <t>12:34</t>
+          <t>12:25</t>
         </is>
       </c>
       <c r="R19" s="6" t="inlineStr">
@@ -2309,17 +2321,17 @@
       </c>
       <c r="S19" s="6" t="inlineStr">
         <is>
-          <t>00:23</t>
+          <t>00:02</t>
         </is>
       </c>
       <c r="T19" s="6" t="inlineStr">
         <is>
-          <t>04:23</t>
+          <t>00:02</t>
         </is>
       </c>
       <c r="U19" s="6" t="inlineStr">
         <is>
-          <t>Imagen de cara</t>
+          <t>Huella dactilar</t>
         </is>
       </c>
       <c r="V19" s="6" t="inlineStr">
@@ -2332,17 +2344,17 @@
     <row r="20" ht="20" customHeight="1">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>44955960</t>
+          <t>44196392</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>ESPINOZA SAAVEDRA</t>
+          <t>BERMEO SANTOS</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>RAUL ESTEBAN</t>
+          <t>ALEXANDER</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
@@ -2352,7 +2364,7 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>COMUNICACIONES</t>
+          <t>MANTENIMIENTO</t>
         </is>
       </c>
       <c r="F20" s="6" t="inlineStr">
@@ -2377,7 +2389,7 @@
       </c>
       <c r="J20" s="6" t="inlineStr">
         <is>
-          <t>07:11</t>
+          <t>06:35</t>
         </is>
       </c>
       <c r="K20" s="6" t="inlineStr">
@@ -2387,17 +2399,17 @@
       </c>
       <c r="L20" s="6" t="inlineStr">
         <is>
-          <t>19:14</t>
+          <t>18:54</t>
         </is>
       </c>
       <c r="M20" s="6" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N20" s="6" t="inlineStr">
         <is>
-          <t>19:33</t>
+          <t>-</t>
         </is>
       </c>
       <c r="O20" s="6" t="inlineStr">
@@ -2412,7 +2424,7 @@
       </c>
       <c r="Q20" s="6" t="inlineStr">
         <is>
-          <t>12:03</t>
+          <t>12:19</t>
         </is>
       </c>
       <c r="R20" s="6" t="inlineStr">
@@ -2422,17 +2434,17 @@
       </c>
       <c r="S20" s="6" t="inlineStr">
         <is>
-          <t>00:14</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="T20" s="6" t="inlineStr">
         <is>
-          <t>00:14</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="U20" s="6" t="inlineStr">
         <is>
-          <t>Imagen de cara</t>
+          <t>Huella dactilar</t>
         </is>
       </c>
       <c r="V20" s="6" t="inlineStr">
@@ -2445,17 +2457,17 @@
     <row r="21" ht="20" customHeight="1">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>45119078</t>
+          <t>44955960</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>CURINAMBE SANCHEZ</t>
+          <t>ESPINOZA SAAVEDRA</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>JOSELITO</t>
+          <t>RAUL ESTEBAN</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
@@ -2465,7 +2477,7 @@
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>OPERACIONES</t>
+          <t>COMUNICACIONES</t>
         </is>
       </c>
       <c r="F21" s="6" t="inlineStr">
@@ -2490,7 +2502,7 @@
       </c>
       <c r="J21" s="6" t="inlineStr">
         <is>
-          <t>07:03</t>
+          <t>06:49</t>
         </is>
       </c>
       <c r="K21" s="6" t="inlineStr">
@@ -2500,32 +2512,32 @@
       </c>
       <c r="L21" s="6" t="inlineStr">
         <is>
-          <t>19:02</t>
+          <t>19:23</t>
         </is>
       </c>
       <c r="M21" s="6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="N21" s="6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>19:48</t>
         </is>
       </c>
       <c r="O21" s="6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="P21" s="6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>23:48</t>
         </is>
       </c>
       <c r="Q21" s="6" t="inlineStr">
         <is>
-          <t>11:59</t>
+          <t>12:34</t>
         </is>
       </c>
       <c r="R21" s="6" t="inlineStr">
@@ -2535,17 +2547,17 @@
       </c>
       <c r="S21" s="6" t="inlineStr">
         <is>
-          <t>00:02</t>
+          <t>00:23</t>
         </is>
       </c>
       <c r="T21" s="6" t="inlineStr">
         <is>
-          <t>00:02</t>
+          <t>04:23</t>
         </is>
       </c>
       <c r="U21" s="6" t="inlineStr">
         <is>
-          <t>Huella dactilar</t>
+          <t>Imagen de cara</t>
         </is>
       </c>
       <c r="V21" s="6" t="inlineStr">
@@ -2558,17 +2570,17 @@
     <row r="22" ht="20" customHeight="1">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>45119078</t>
+          <t>44955960</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>CURINAMBE SANCHEZ</t>
+          <t>ESPINOZA SAAVEDRA</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>JOSELITO</t>
+          <t>RAUL ESTEBAN</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
@@ -2578,7 +2590,7 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>OPERACIONES</t>
+          <t>COMUNICACIONES</t>
         </is>
       </c>
       <c r="F22" s="6" t="inlineStr">
@@ -2603,7 +2615,7 @@
       </c>
       <c r="J22" s="6" t="inlineStr">
         <is>
-          <t>06:42</t>
+          <t>07:11</t>
         </is>
       </c>
       <c r="K22" s="6" t="inlineStr">
@@ -2613,17 +2625,17 @@
       </c>
       <c r="L22" s="6" t="inlineStr">
         <is>
-          <t>19:11</t>
+          <t>19:14</t>
         </is>
       </c>
       <c r="M22" s="6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="N22" s="6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>19:33</t>
         </is>
       </c>
       <c r="O22" s="6" t="inlineStr">
@@ -2638,7 +2650,7 @@
       </c>
       <c r="Q22" s="6" t="inlineStr">
         <is>
-          <t>12:29</t>
+          <t>12:03</t>
         </is>
       </c>
       <c r="R22" s="6" t="inlineStr">
@@ -2648,17 +2660,17 @@
       </c>
       <c r="S22" s="6" t="inlineStr">
         <is>
-          <t>00:11</t>
+          <t>00:14</t>
         </is>
       </c>
       <c r="T22" s="6" t="inlineStr">
         <is>
-          <t>00:11</t>
+          <t>00:14</t>
         </is>
       </c>
       <c r="U22" s="6" t="inlineStr">
         <is>
-          <t>Huella dactilar</t>
+          <t>Imagen de cara</t>
         </is>
       </c>
       <c r="V22" s="6" t="inlineStr">
@@ -2671,27 +2683,27 @@
     <row r="23" ht="20" customHeight="1">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>47034929</t>
+          <t>45119078</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>ALVA MEDINA</t>
+          <t>CURINAMBE SANCHEZ</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>JHON KENEDY</t>
+          <t>JOSELITO</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>JEFATURA</t>
+          <t>OPER&amp;MTTO</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t>JEFE</t>
+          <t>OPERACIONES</t>
         </is>
       </c>
       <c r="F23" s="6" t="inlineStr">
@@ -2716,7 +2728,7 @@
       </c>
       <c r="J23" s="6" t="inlineStr">
         <is>
-          <t>07:05</t>
+          <t>07:03</t>
         </is>
       </c>
       <c r="K23" s="6" t="inlineStr">
@@ -2726,7 +2738,7 @@
       </c>
       <c r="L23" s="6" t="inlineStr">
         <is>
-          <t>19:22</t>
+          <t>19:02</t>
         </is>
       </c>
       <c r="M23" s="6" t="inlineStr">
@@ -2751,7 +2763,7 @@
       </c>
       <c r="Q23" s="6" t="inlineStr">
         <is>
-          <t>12:17</t>
+          <t>11:59</t>
         </is>
       </c>
       <c r="R23" s="6" t="inlineStr">
@@ -2761,12 +2773,12 @@
       </c>
       <c r="S23" s="6" t="inlineStr">
         <is>
-          <t>00:22</t>
+          <t>00:02</t>
         </is>
       </c>
       <c r="T23" s="6" t="inlineStr">
         <is>
-          <t>00:22</t>
+          <t>00:02</t>
         </is>
       </c>
       <c r="U23" s="6" t="inlineStr">
@@ -2784,27 +2796,27 @@
     <row r="24" ht="20" customHeight="1">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>47034929</t>
+          <t>45119078</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>ALVA MEDINA</t>
+          <t>CURINAMBE SANCHEZ</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>JHON KENEDY</t>
+          <t>JOSELITO</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>JEFATURA</t>
+          <t>OPER&amp;MTTO</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>JEFE</t>
+          <t>OPERACIONES</t>
         </is>
       </c>
       <c r="F24" s="6" t="inlineStr">
@@ -2829,7 +2841,7 @@
       </c>
       <c r="J24" s="6" t="inlineStr">
         <is>
-          <t>07:17</t>
+          <t>06:42</t>
         </is>
       </c>
       <c r="K24" s="6" t="inlineStr">
@@ -2839,7 +2851,7 @@
       </c>
       <c r="L24" s="6" t="inlineStr">
         <is>
-          <t>20:27</t>
+          <t>19:11</t>
         </is>
       </c>
       <c r="M24" s="6" t="inlineStr">
@@ -2864,27 +2876,27 @@
       </c>
       <c r="Q24" s="6" t="inlineStr">
         <is>
-          <t>13:10</t>
+          <t>12:29</t>
         </is>
       </c>
       <c r="R24" s="6" t="inlineStr">
         <is>
-          <t>00:02</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="S24" s="6" t="inlineStr">
         <is>
-          <t>01:27</t>
+          <t>00:11</t>
         </is>
       </c>
       <c r="T24" s="6" t="inlineStr">
         <is>
-          <t>01:27</t>
+          <t>00:11</t>
         </is>
       </c>
       <c r="U24" s="6" t="inlineStr">
         <is>
-          <t>Imagen de cara</t>
+          <t>Huella dactilar</t>
         </is>
       </c>
       <c r="V24" s="6" t="inlineStr">
@@ -2892,36 +2904,32 @@
           <t>Normal</t>
         </is>
       </c>
-      <c r="W24" s="5" t="inlineStr">
-        <is>
-          <t>Tardanza (2 min), Exceso de jornada no autorizado (87 min)</t>
-        </is>
-      </c>
+      <c r="W24" s="5" t="inlineStr"/>
     </row>
     <row r="25" ht="20" customHeight="1">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>47591578</t>
+          <t>47034929</t>
         </is>
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>NINAQUISPE JACOBO</t>
+          <t>ALVA MEDINA</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>LUIS MIGUEL</t>
+          <t>JHON KENEDY</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>OPER&amp;MTTO</t>
+          <t>JEFATURA</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t>OPERACIONES</t>
+          <t>JEFE</t>
         </is>
       </c>
       <c r="F25" s="6" t="inlineStr">
@@ -2946,7 +2954,7 @@
       </c>
       <c r="J25" s="6" t="inlineStr">
         <is>
-          <t>06:44</t>
+          <t>07:05</t>
         </is>
       </c>
       <c r="K25" s="6" t="inlineStr">
@@ -2956,7 +2964,7 @@
       </c>
       <c r="L25" s="6" t="inlineStr">
         <is>
-          <t>19:15</t>
+          <t>19:22</t>
         </is>
       </c>
       <c r="M25" s="6" t="inlineStr">
@@ -2981,7 +2989,7 @@
       </c>
       <c r="Q25" s="6" t="inlineStr">
         <is>
-          <t>12:31</t>
+          <t>12:17</t>
         </is>
       </c>
       <c r="R25" s="6" t="inlineStr">
@@ -2991,17 +2999,17 @@
       </c>
       <c r="S25" s="6" t="inlineStr">
         <is>
-          <t>00:15</t>
+          <t>00:22</t>
         </is>
       </c>
       <c r="T25" s="6" t="inlineStr">
         <is>
-          <t>00:15</t>
+          <t>00:22</t>
         </is>
       </c>
       <c r="U25" s="6" t="inlineStr">
         <is>
-          <t>Imagen de cara</t>
+          <t>Huella dactilar</t>
         </is>
       </c>
       <c r="V25" s="6" t="inlineStr">
@@ -3014,27 +3022,27 @@
     <row r="26" ht="20" customHeight="1">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>47591578</t>
+          <t>47034929</t>
         </is>
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>NINAQUISPE JACOBO</t>
+          <t>ALVA MEDINA</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>LUIS MIGUEL</t>
+          <t>JHON KENEDY</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>OPER&amp;MTTO</t>
+          <t>JEFATURA</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t>OPERACIONES</t>
+          <t>JEFE</t>
         </is>
       </c>
       <c r="F26" s="6" t="inlineStr">
@@ -3059,7 +3067,7 @@
       </c>
       <c r="J26" s="6" t="inlineStr">
         <is>
-          <t>07:12</t>
+          <t>07:17</t>
         </is>
       </c>
       <c r="K26" s="6" t="inlineStr">
@@ -3069,7 +3077,7 @@
       </c>
       <c r="L26" s="6" t="inlineStr">
         <is>
-          <t>18:56</t>
+          <t>20:27</t>
         </is>
       </c>
       <c r="M26" s="6" t="inlineStr">
@@ -3094,22 +3102,22 @@
       </c>
       <c r="Q26" s="6" t="inlineStr">
         <is>
-          <t>11:44</t>
+          <t>13:10</t>
         </is>
       </c>
       <c r="R26" s="6" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>00:02</t>
         </is>
       </c>
       <c r="S26" s="6" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>01:27</t>
         </is>
       </c>
       <c r="T26" s="6" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>01:27</t>
         </is>
       </c>
       <c r="U26" s="6" t="inlineStr">
@@ -3122,22 +3130,26 @@
           <t>Normal</t>
         </is>
       </c>
-      <c r="W26" s="5" t="inlineStr"/>
+      <c r="W26" s="5" t="inlineStr">
+        <is>
+          <t>Tardanza (2 min), Exceso de jornada no autorizado (87 min)</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="20" customHeight="1">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>47721216</t>
+          <t>47591578</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>SANCHEZ RAMIREZ</t>
+          <t>NINAQUISPE JACOBO</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>PAUL JAIR</t>
+          <t>LUIS MIGUEL</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
@@ -3172,7 +3184,7 @@
       </c>
       <c r="J27" s="6" t="inlineStr">
         <is>
-          <t>06:46</t>
+          <t>06:44</t>
         </is>
       </c>
       <c r="K27" s="6" t="inlineStr">
@@ -3182,7 +3194,7 @@
       </c>
       <c r="L27" s="6" t="inlineStr">
         <is>
-          <t>19:04</t>
+          <t>19:15</t>
         </is>
       </c>
       <c r="M27" s="6" t="inlineStr">
@@ -3207,7 +3219,7 @@
       </c>
       <c r="Q27" s="6" t="inlineStr">
         <is>
-          <t>12:18</t>
+          <t>12:31</t>
         </is>
       </c>
       <c r="R27" s="6" t="inlineStr">
@@ -3217,17 +3229,17 @@
       </c>
       <c r="S27" s="6" t="inlineStr">
         <is>
-          <t>00:04</t>
+          <t>00:15</t>
         </is>
       </c>
       <c r="T27" s="6" t="inlineStr">
         <is>
-          <t>00:04</t>
+          <t>00:15</t>
         </is>
       </c>
       <c r="U27" s="6" t="inlineStr">
         <is>
-          <t>Huella dactilar</t>
+          <t>Imagen de cara</t>
         </is>
       </c>
       <c r="V27" s="6" t="inlineStr">
@@ -3240,17 +3252,17 @@
     <row r="28" ht="20" customHeight="1">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>47721216</t>
+          <t>47591578</t>
         </is>
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>SANCHEZ RAMIREZ</t>
+          <t>NINAQUISPE JACOBO</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>PAUL JAIR</t>
+          <t>LUIS MIGUEL</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
@@ -3285,7 +3297,7 @@
       </c>
       <c r="J28" s="6" t="inlineStr">
         <is>
-          <t>06:40</t>
+          <t>07:12</t>
         </is>
       </c>
       <c r="K28" s="6" t="inlineStr">
@@ -3295,7 +3307,7 @@
       </c>
       <c r="L28" s="6" t="inlineStr">
         <is>
-          <t>21:42</t>
+          <t>18:56</t>
         </is>
       </c>
       <c r="M28" s="6" t="inlineStr">
@@ -3320,7 +3332,7 @@
       </c>
       <c r="Q28" s="6" t="inlineStr">
         <is>
-          <t>15:02</t>
+          <t>11:44</t>
         </is>
       </c>
       <c r="R28" s="6" t="inlineStr">
@@ -3330,12 +3342,12 @@
       </c>
       <c r="S28" s="6" t="inlineStr">
         <is>
-          <t>02:42</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="T28" s="6" t="inlineStr">
         <is>
-          <t>02:42</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="U28" s="6" t="inlineStr">
@@ -3348,26 +3360,22 @@
           <t>Normal</t>
         </is>
       </c>
-      <c r="W28" s="5" t="inlineStr">
-        <is>
-          <t>Exceso de jornada no autorizado (162 min)</t>
-        </is>
-      </c>
+      <c r="W28" s="5" t="inlineStr"/>
     </row>
     <row r="29" ht="20" customHeight="1">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>47783594</t>
+          <t>47721216</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>AGREDA ASPAJO</t>
+          <t>SANCHEZ RAMIREZ</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>JHON ROBERT</t>
+          <t>PAUL JAIR</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
@@ -3377,7 +3385,7 @@
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t>MAESTRANZA</t>
+          <t>OPERACIONES</t>
         </is>
       </c>
       <c r="F29" s="6" t="inlineStr">
@@ -3402,7 +3410,7 @@
       </c>
       <c r="J29" s="6" t="inlineStr">
         <is>
-          <t>07:05</t>
+          <t>06:46</t>
         </is>
       </c>
       <c r="K29" s="6" t="inlineStr">
@@ -3412,7 +3420,7 @@
       </c>
       <c r="L29" s="6" t="inlineStr">
         <is>
-          <t>20:16</t>
+          <t>19:04</t>
         </is>
       </c>
       <c r="M29" s="6" t="inlineStr">
@@ -3437,7 +3445,7 @@
       </c>
       <c r="Q29" s="6" t="inlineStr">
         <is>
-          <t>13:11</t>
+          <t>12:18</t>
         </is>
       </c>
       <c r="R29" s="6" t="inlineStr">
@@ -3447,12 +3455,12 @@
       </c>
       <c r="S29" s="6" t="inlineStr">
         <is>
-          <t>01:16</t>
+          <t>00:04</t>
         </is>
       </c>
       <c r="T29" s="6" t="inlineStr">
         <is>
-          <t>01:16</t>
+          <t>00:04</t>
         </is>
       </c>
       <c r="U29" s="6" t="inlineStr">
@@ -3462,29 +3470,25 @@
       </c>
       <c r="V29" s="6" t="inlineStr">
         <is>
-          <t>Duplicado (Entrada)</t>
-        </is>
-      </c>
-      <c r="W29" s="5" t="inlineStr">
-        <is>
-          <t>Entrada duplicada (20:16), Exceso de jornada no autorizado (76 min)</t>
-        </is>
-      </c>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="W29" s="5" t="inlineStr"/>
     </row>
     <row r="30" ht="20" customHeight="1">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>47783594</t>
+          <t>47721216</t>
         </is>
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>AGREDA ASPAJO</t>
+          <t>SANCHEZ RAMIREZ</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>JHON ROBERT</t>
+          <t>PAUL JAIR</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
@@ -3494,7 +3498,7 @@
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t>MAESTRANZA</t>
+          <t>OPERACIONES</t>
         </is>
       </c>
       <c r="F30" s="6" t="inlineStr">
@@ -3519,7 +3523,7 @@
       </c>
       <c r="J30" s="6" t="inlineStr">
         <is>
-          <t>07:12</t>
+          <t>06:40</t>
         </is>
       </c>
       <c r="K30" s="6" t="inlineStr">
@@ -3529,7 +3533,7 @@
       </c>
       <c r="L30" s="6" t="inlineStr">
         <is>
-          <t>20:23</t>
+          <t>21:42</t>
         </is>
       </c>
       <c r="M30" s="6" t="inlineStr">
@@ -3554,7 +3558,7 @@
       </c>
       <c r="Q30" s="6" t="inlineStr">
         <is>
-          <t>13:11</t>
+          <t>15:02</t>
         </is>
       </c>
       <c r="R30" s="6" t="inlineStr">
@@ -3564,17 +3568,17 @@
       </c>
       <c r="S30" s="6" t="inlineStr">
         <is>
-          <t>01:23</t>
+          <t>02:42</t>
         </is>
       </c>
       <c r="T30" s="6" t="inlineStr">
         <is>
-          <t>01:23</t>
+          <t>02:42</t>
         </is>
       </c>
       <c r="U30" s="6" t="inlineStr">
         <is>
-          <t>Huella dactilar</t>
+          <t>Imagen de cara</t>
         </is>
       </c>
       <c r="V30" s="6" t="inlineStr">
@@ -3584,34 +3588,34 @@
       </c>
       <c r="W30" s="5" t="inlineStr">
         <is>
-          <t>Exceso de jornada no autorizado (83 min)</t>
+          <t>Exceso de jornada no autorizado (162 min)</t>
         </is>
       </c>
     </row>
     <row r="31" ht="20" customHeight="1">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>48455175</t>
+          <t>47783594</t>
         </is>
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>VASQUEZ PUELLES</t>
+          <t>AGREDA ASPAJO</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>IVAN ANTONIO</t>
+          <t>JHON ROBERT</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>ADMINISTRACIÓN</t>
+          <t>OPER&amp;MTTO</t>
         </is>
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO</t>
+          <t>MAESTRANZA</t>
         </is>
       </c>
       <c r="F31" s="6" t="inlineStr">
@@ -3636,11 +3640,19 @@
       </c>
       <c r="J31" s="6" t="inlineStr">
         <is>
-          <t>07:20</t>
-        </is>
-      </c>
-      <c r="K31" s="6" t="inlineStr"/>
-      <c r="L31" s="6" t="inlineStr"/>
+          <t>07:05</t>
+        </is>
+      </c>
+      <c r="K31" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="L31" s="6" t="inlineStr">
+        <is>
+          <t>20:16</t>
+        </is>
+      </c>
       <c r="M31" s="6" t="inlineStr">
         <is>
           <t>-</t>
@@ -3663,64 +3675,64 @@
       </c>
       <c r="Q31" s="6" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>13:11</t>
         </is>
       </c>
       <c r="R31" s="6" t="inlineStr">
         <is>
-          <t>00:05</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="S31" s="6" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>01:16</t>
         </is>
       </c>
       <c r="T31" s="6" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>01:16</t>
         </is>
       </c>
       <c r="U31" s="6" t="inlineStr">
         <is>
-          <t>Imagen de cara</t>
+          <t>Huella dactilar</t>
         </is>
       </c>
       <c r="V31" s="6" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>Duplicado (Entrada)</t>
         </is>
       </c>
       <c r="W31" s="5" t="inlineStr">
         <is>
-          <t>Falta marcación de salida, Tardanza (5 min)</t>
+          <t>Entrada duplicada (20:16), Exceso de jornada no autorizado (76 min)</t>
         </is>
       </c>
     </row>
     <row r="32" ht="20" customHeight="1">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>48455175</t>
+          <t>47783594</t>
         </is>
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>VASQUEZ PUELLES</t>
+          <t>AGREDA ASPAJO</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>IVAN ANTONIO</t>
+          <t>JHON ROBERT</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>ADMINISTRACIÓN</t>
+          <t>OPER&amp;MTTO</t>
         </is>
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO</t>
+          <t>MAESTRANZA</t>
         </is>
       </c>
       <c r="F32" s="6" t="inlineStr">
@@ -3745,7 +3757,7 @@
       </c>
       <c r="J32" s="6" t="inlineStr">
         <is>
-          <t>06:41</t>
+          <t>07:12</t>
         </is>
       </c>
       <c r="K32" s="6" t="inlineStr">
@@ -3755,7 +3767,7 @@
       </c>
       <c r="L32" s="6" t="inlineStr">
         <is>
-          <t>19:01</t>
+          <t>20:23</t>
         </is>
       </c>
       <c r="M32" s="6" t="inlineStr">
@@ -3780,7 +3792,7 @@
       </c>
       <c r="Q32" s="6" t="inlineStr">
         <is>
-          <t>12:20</t>
+          <t>13:11</t>
         </is>
       </c>
       <c r="R32" s="6" t="inlineStr">
@@ -3790,12 +3802,12 @@
       </c>
       <c r="S32" s="6" t="inlineStr">
         <is>
-          <t>00:01</t>
+          <t>01:23</t>
         </is>
       </c>
       <c r="T32" s="6" t="inlineStr">
         <is>
-          <t>00:01</t>
+          <t>01:23</t>
         </is>
       </c>
       <c r="U32" s="6" t="inlineStr">
@@ -3805,39 +3817,39 @@
       </c>
       <c r="V32" s="6" t="inlineStr">
         <is>
-          <t>Duplicado (Entrada)</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="W32" s="5" t="inlineStr">
         <is>
-          <t>Entrada duplicada (19:01)</t>
+          <t>Exceso de jornada no autorizado (83 min)</t>
         </is>
       </c>
     </row>
     <row r="33" ht="20" customHeight="1">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>48790853</t>
+          <t>48455175</t>
         </is>
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>GUERRA SAJAMI</t>
+          <t>VASQUEZ PUELLES</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>SANGABIL</t>
+          <t>IVAN ANTONIO</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
         <is>
-          <t>OPER&amp;MTTO</t>
+          <t>ADMINISTRACIÓN</t>
         </is>
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t>OPERACIONES</t>
+          <t>ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="F33" s="6" t="inlineStr">
@@ -3852,7 +3864,7 @@
       </c>
       <c r="H33" s="6" t="inlineStr">
         <is>
-          <t>NOCHE</t>
+          <t>DIA</t>
         </is>
       </c>
       <c r="I33" s="6" t="inlineStr">
@@ -3862,7 +3874,7 @@
       </c>
       <c r="J33" s="6" t="inlineStr">
         <is>
-          <t>18:50</t>
+          <t>07:20</t>
         </is>
       </c>
       <c r="K33" s="6" t="inlineStr"/>
@@ -3894,7 +3906,7 @@
       </c>
       <c r="R33" s="6" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>00:05</t>
         </is>
       </c>
       <c r="S33" s="6" t="inlineStr">
@@ -3909,7 +3921,7 @@
       </c>
       <c r="U33" s="6" t="inlineStr">
         <is>
-          <t>Huella dactilar</t>
+          <t>Imagen de cara</t>
         </is>
       </c>
       <c r="V33" s="6" t="inlineStr">
@@ -3919,34 +3931,34 @@
       </c>
       <c r="W33" s="5" t="inlineStr">
         <is>
-          <t>Falta marcación de salida</t>
+          <t>Falta marcación de salida, Tardanza (5 min)</t>
         </is>
       </c>
     </row>
     <row r="34" ht="20" customHeight="1">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t>48790853</t>
+          <t>48455175</t>
         </is>
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>GUERRA SAJAMI</t>
+          <t>VASQUEZ PUELLES</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>SANGABIL</t>
+          <t>IVAN ANTONIO</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>OPER&amp;MTTO</t>
+          <t>ADMINISTRACIÓN</t>
         </is>
       </c>
       <c r="E34" s="5" t="inlineStr">
         <is>
-          <t>OPERACIONES</t>
+          <t>ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="F34" s="6" t="inlineStr">
@@ -3961,7 +3973,7 @@
       </c>
       <c r="H34" s="6" t="inlineStr">
         <is>
-          <t>NOCHE</t>
+          <t>DIA</t>
         </is>
       </c>
       <c r="I34" s="6" t="inlineStr">
@@ -3971,7 +3983,7 @@
       </c>
       <c r="J34" s="6" t="inlineStr">
         <is>
-          <t>18:40</t>
+          <t>06:41</t>
         </is>
       </c>
       <c r="K34" s="6" t="inlineStr">
@@ -3981,7 +3993,7 @@
       </c>
       <c r="L34" s="6" t="inlineStr">
         <is>
-          <t>07:01</t>
+          <t>19:01</t>
         </is>
       </c>
       <c r="M34" s="6" t="inlineStr">
@@ -4006,7 +4018,7 @@
       </c>
       <c r="Q34" s="6" t="inlineStr">
         <is>
-          <t>12:21</t>
+          <t>12:20</t>
         </is>
       </c>
       <c r="R34" s="6" t="inlineStr">
@@ -4026,30 +4038,34 @@
       </c>
       <c r="U34" s="6" t="inlineStr">
         <is>
-          <t>Imagen de cara</t>
+          <t>Huella dactilar</t>
         </is>
       </c>
       <c r="V34" s="6" t="inlineStr">
         <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="W34" s="5" t="inlineStr"/>
+          <t>Duplicado (Entrada)</t>
+        </is>
+      </c>
+      <c r="W34" s="5" t="inlineStr">
+        <is>
+          <t>Entrada duplicada (19:01)</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="20" customHeight="1">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t>60512609</t>
+          <t>48790853</t>
         </is>
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>SUAREZ CAMPOS</t>
+          <t>GUERRA SAJAMI</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>EDERLY</t>
+          <t>SANGABIL</t>
         </is>
       </c>
       <c r="D35" s="5" t="inlineStr">
@@ -4074,7 +4090,7 @@
       </c>
       <c r="H35" s="6" t="inlineStr">
         <is>
-          <t>DIA</t>
+          <t>NOCHE</t>
         </is>
       </c>
       <c r="I35" s="6" t="inlineStr">
@@ -4084,19 +4100,11 @@
       </c>
       <c r="J35" s="6" t="inlineStr">
         <is>
-          <t>06:43</t>
-        </is>
-      </c>
-      <c r="K35" s="6" t="inlineStr">
-        <is>
-          <t>2026-08-17</t>
-        </is>
-      </c>
-      <c r="L35" s="6" t="inlineStr">
-        <is>
-          <t>20:18</t>
-        </is>
-      </c>
+          <t>18:50</t>
+        </is>
+      </c>
+      <c r="K35" s="6" t="inlineStr"/>
+      <c r="L35" s="6" t="inlineStr"/>
       <c r="M35" s="6" t="inlineStr">
         <is>
           <t>-</t>
@@ -4119,7 +4127,7 @@
       </c>
       <c r="Q35" s="6" t="inlineStr">
         <is>
-          <t>13:35</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="R35" s="6" t="inlineStr">
@@ -4129,12 +4137,12 @@
       </c>
       <c r="S35" s="6" t="inlineStr">
         <is>
-          <t>01:18</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="T35" s="6" t="inlineStr">
         <is>
-          <t>01:18</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="U35" s="6" t="inlineStr">
@@ -4144,29 +4152,29 @@
       </c>
       <c r="V35" s="6" t="inlineStr">
         <is>
-          <t>Duplicado (Entrada)</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="W35" s="5" t="inlineStr">
         <is>
-          <t>Entrada duplicada (20:16), Exceso de jornada no autorizado (78 min)</t>
+          <t>Falta marcación de salida</t>
         </is>
       </c>
     </row>
     <row r="36" ht="20" customHeight="1">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t>60512609</t>
+          <t>48790853</t>
         </is>
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>SUAREZ CAMPOS</t>
+          <t>GUERRA SAJAMI</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>EDERLY</t>
+          <t>SANGABIL</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
@@ -4191,7 +4199,7 @@
       </c>
       <c r="H36" s="6" t="inlineStr">
         <is>
-          <t>DIA</t>
+          <t>NOCHE</t>
         </is>
       </c>
       <c r="I36" s="6" t="inlineStr">
@@ -4201,7 +4209,7 @@
       </c>
       <c r="J36" s="6" t="inlineStr">
         <is>
-          <t>06:39</t>
+          <t>18:40</t>
         </is>
       </c>
       <c r="K36" s="6" t="inlineStr">
@@ -4211,7 +4219,7 @@
       </c>
       <c r="L36" s="6" t="inlineStr">
         <is>
-          <t>21:38</t>
+          <t>07:01</t>
         </is>
       </c>
       <c r="M36" s="6" t="inlineStr">
@@ -4236,7 +4244,7 @@
       </c>
       <c r="Q36" s="6" t="inlineStr">
         <is>
-          <t>14:59</t>
+          <t>12:21</t>
         </is>
       </c>
       <c r="R36" s="6" t="inlineStr">
@@ -4246,17 +4254,17 @@
       </c>
       <c r="S36" s="6" t="inlineStr">
         <is>
-          <t>02:38</t>
+          <t>00:01</t>
         </is>
       </c>
       <c r="T36" s="6" t="inlineStr">
         <is>
-          <t>02:38</t>
+          <t>00:01</t>
         </is>
       </c>
       <c r="U36" s="6" t="inlineStr">
         <is>
-          <t>Huella dactilar</t>
+          <t>Imagen de cara</t>
         </is>
       </c>
       <c r="V36" s="6" t="inlineStr">
@@ -4264,26 +4272,22 @@
           <t>Normal</t>
         </is>
       </c>
-      <c r="W36" s="5" t="inlineStr">
-        <is>
-          <t>Exceso de jornada no autorizado (158 min)</t>
-        </is>
-      </c>
+      <c r="W36" s="5" t="inlineStr"/>
     </row>
     <row r="37" ht="20" customHeight="1">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>60876523</t>
+          <t>60512609</t>
         </is>
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>ALBITRES GONZALES</t>
+          <t>SUAREZ CAMPOS</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>DEYVI</t>
+          <t>EDERLY</t>
         </is>
       </c>
       <c r="D37" s="5" t="inlineStr">
@@ -4293,7 +4297,7 @@
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t>MAQUINARIA PESADA</t>
+          <t>OPERACIONES</t>
         </is>
       </c>
       <c r="F37" s="6" t="inlineStr">
@@ -4308,7 +4312,7 @@
       </c>
       <c r="H37" s="6" t="inlineStr">
         <is>
-          <t>NOCHE</t>
+          <t>DIA</t>
         </is>
       </c>
       <c r="I37" s="6" t="inlineStr">
@@ -4318,11 +4322,19 @@
       </c>
       <c r="J37" s="6" t="inlineStr">
         <is>
-          <t>18:32</t>
-        </is>
-      </c>
-      <c r="K37" s="6" t="inlineStr"/>
-      <c r="L37" s="6" t="inlineStr"/>
+          <t>06:43</t>
+        </is>
+      </c>
+      <c r="K37" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="L37" s="6" t="inlineStr">
+        <is>
+          <t>20:18</t>
+        </is>
+      </c>
       <c r="M37" s="6" t="inlineStr">
         <is>
           <t>-</t>
@@ -4345,7 +4357,7 @@
       </c>
       <c r="Q37" s="6" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>13:35</t>
         </is>
       </c>
       <c r="R37" s="6" t="inlineStr">
@@ -4355,12 +4367,12 @@
       </c>
       <c r="S37" s="6" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>01:18</t>
         </is>
       </c>
       <c r="T37" s="6" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>01:18</t>
         </is>
       </c>
       <c r="U37" s="6" t="inlineStr">
@@ -4370,29 +4382,29 @@
       </c>
       <c r="V37" s="6" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>Duplicado (Entrada)</t>
         </is>
       </c>
       <c r="W37" s="5" t="inlineStr">
         <is>
-          <t>Falta marcación de salida</t>
+          <t>Entrada duplicada (20:16), Exceso de jornada no autorizado (78 min)</t>
         </is>
       </c>
     </row>
     <row r="38" ht="20" customHeight="1">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>60876523</t>
+          <t>60512609</t>
         </is>
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>ALBITRES GONZALES</t>
+          <t>SUAREZ CAMPOS</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>DEYVI</t>
+          <t>EDERLY</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
@@ -4402,7 +4414,7 @@
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t>MAQUINARIA PESADA</t>
+          <t>OPERACIONES</t>
         </is>
       </c>
       <c r="F38" s="6" t="inlineStr">
@@ -4417,7 +4429,7 @@
       </c>
       <c r="H38" s="6" t="inlineStr">
         <is>
-          <t>NOCHE</t>
+          <t>DIA</t>
         </is>
       </c>
       <c r="I38" s="6" t="inlineStr">
@@ -4427,7 +4439,7 @@
       </c>
       <c r="J38" s="6" t="inlineStr">
         <is>
-          <t>18:31</t>
+          <t>06:39</t>
         </is>
       </c>
       <c r="K38" s="6" t="inlineStr">
@@ -4437,7 +4449,7 @@
       </c>
       <c r="L38" s="6" t="inlineStr">
         <is>
-          <t>07:01</t>
+          <t>21:38</t>
         </is>
       </c>
       <c r="M38" s="6" t="inlineStr">
@@ -4462,7 +4474,7 @@
       </c>
       <c r="Q38" s="6" t="inlineStr">
         <is>
-          <t>12:30</t>
+          <t>14:59</t>
         </is>
       </c>
       <c r="R38" s="6" t="inlineStr">
@@ -4472,12 +4484,12 @@
       </c>
       <c r="S38" s="6" t="inlineStr">
         <is>
-          <t>00:01</t>
+          <t>02:38</t>
         </is>
       </c>
       <c r="T38" s="6" t="inlineStr">
         <is>
-          <t>00:01</t>
+          <t>02:38</t>
         </is>
       </c>
       <c r="U38" s="6" t="inlineStr">
@@ -4490,28 +4502,36 @@
           <t>Normal</t>
         </is>
       </c>
-      <c r="W38" s="5" t="inlineStr"/>
+      <c r="W38" s="5" t="inlineStr">
+        <is>
+          <t>Exceso de jornada no autorizado (158 min)</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="20" customHeight="1">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>6616501</t>
+          <t>60876523</t>
         </is>
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>DESCONOCIDO</t>
-        </is>
-      </c>
-      <c r="C39" s="5" t="inlineStr"/>
+          <t>ALBITRES GONZALES</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>DEYVI</t>
+        </is>
+      </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>OPER&amp;MTTO</t>
         </is>
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>MAQUINARIA PESADA</t>
         </is>
       </c>
       <c r="F39" s="6" t="inlineStr">
@@ -4526,7 +4546,7 @@
       </c>
       <c r="H39" s="6" t="inlineStr">
         <is>
-          <t>DIA</t>
+          <t>NOCHE</t>
         </is>
       </c>
       <c r="I39" s="6" t="inlineStr">
@@ -4536,19 +4556,11 @@
       </c>
       <c r="J39" s="6" t="inlineStr">
         <is>
-          <t>06:49</t>
-        </is>
-      </c>
-      <c r="K39" s="6" t="inlineStr">
-        <is>
-          <t>2026-08-17</t>
-        </is>
-      </c>
-      <c r="L39" s="6" t="inlineStr">
-        <is>
-          <t>20:17</t>
-        </is>
-      </c>
+          <t>18:32</t>
+        </is>
+      </c>
+      <c r="K39" s="6" t="inlineStr"/>
+      <c r="L39" s="6" t="inlineStr"/>
       <c r="M39" s="6" t="inlineStr">
         <is>
           <t>-</t>
@@ -4571,7 +4583,7 @@
       </c>
       <c r="Q39" s="6" t="inlineStr">
         <is>
-          <t>13:28</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="R39" s="6" t="inlineStr">
@@ -4581,12 +4593,12 @@
       </c>
       <c r="S39" s="6" t="inlineStr">
         <is>
-          <t>01:17</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="T39" s="6" t="inlineStr">
         <is>
-          <t>01:17</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="U39" s="6" t="inlineStr">
@@ -4596,35 +4608,39 @@
       </c>
       <c r="V39" s="6" t="inlineStr">
         <is>
-          <t>Duplicado (Entrada)</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="W39" s="5" t="inlineStr">
         <is>
-          <t>Entrada duplicada (20:15), Exceso de jornada no autorizado (77 min)</t>
+          <t>Falta marcación de salida</t>
         </is>
       </c>
     </row>
     <row r="40" ht="20" customHeight="1">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t>6616501</t>
+          <t>60876523</t>
         </is>
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>DESCONOCIDO</t>
-        </is>
-      </c>
-      <c r="C40" s="5" t="inlineStr"/>
+          <t>ALBITRES GONZALES</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>DEYVI</t>
+        </is>
+      </c>
       <c r="D40" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>OPER&amp;MTTO</t>
         </is>
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>MAQUINARIA PESADA</t>
         </is>
       </c>
       <c r="F40" s="6" t="inlineStr">
@@ -4639,7 +4655,7 @@
       </c>
       <c r="H40" s="6" t="inlineStr">
         <is>
-          <t>DIA</t>
+          <t>NOCHE</t>
         </is>
       </c>
       <c r="I40" s="6" t="inlineStr">
@@ -4649,7 +4665,7 @@
       </c>
       <c r="J40" s="6" t="inlineStr">
         <is>
-          <t>06:41</t>
+          <t>18:31</t>
         </is>
       </c>
       <c r="K40" s="6" t="inlineStr">
@@ -4659,7 +4675,7 @@
       </c>
       <c r="L40" s="6" t="inlineStr">
         <is>
-          <t>21:37</t>
+          <t>07:01</t>
         </is>
       </c>
       <c r="M40" s="6" t="inlineStr">
@@ -4684,7 +4700,7 @@
       </c>
       <c r="Q40" s="6" t="inlineStr">
         <is>
-          <t>14:56</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="R40" s="6" t="inlineStr">
@@ -4694,17 +4710,17 @@
       </c>
       <c r="S40" s="6" t="inlineStr">
         <is>
-          <t>02:37</t>
+          <t>00:01</t>
         </is>
       </c>
       <c r="T40" s="6" t="inlineStr">
         <is>
-          <t>02:37</t>
+          <t>00:01</t>
         </is>
       </c>
       <c r="U40" s="6" t="inlineStr">
         <is>
-          <t>Imagen de cara</t>
+          <t>Huella dactilar</t>
         </is>
       </c>
       <c r="V40" s="6" t="inlineStr">
@@ -4712,11 +4728,7 @@
           <t>Normal</t>
         </is>
       </c>
-      <c r="W40" s="5" t="inlineStr">
-        <is>
-          <t>Exceso de jornada no autorizado (157 min)</t>
-        </is>
-      </c>
+      <c r="W40" s="5" t="inlineStr"/>
     </row>
     <row r="41" ht="20" customHeight="1">
       <c r="A41" s="4" t="inlineStr">
@@ -8651,7 +8663,7 @@
       </c>
       <c r="U75" s="6" t="inlineStr">
         <is>
-          <t>Huella dactilar</t>
+          <t>-</t>
         </is>
       </c>
       <c r="V75" s="6" t="inlineStr">
@@ -8873,7 +8885,7 @@
       </c>
       <c r="U77" s="6" t="inlineStr">
         <is>
-          <t>Huella dactilar</t>
+          <t>-</t>
         </is>
       </c>
       <c r="V77" s="6" t="inlineStr">
@@ -9876,17 +9888,17 @@
     <row r="88" ht="20" customHeight="1">
       <c r="A88" s="4" t="inlineStr">
         <is>
-          <t>006616501</t>
+          <t>71715827</t>
         </is>
       </c>
       <c r="B88" s="5" t="inlineStr">
         <is>
-          <t>ORDOÑEZ ARTEAGA</t>
+          <t>ROJAS CASTRO</t>
         </is>
       </c>
       <c r="C88" s="5" t="inlineStr">
         <is>
-          <t>YENKLI VICENTE</t>
+          <t>ALAN JANDY</t>
         </is>
       </c>
       <c r="D88" s="5" t="inlineStr">
@@ -9896,7 +9908,7 @@
       </c>
       <c r="E88" s="5" t="inlineStr">
         <is>
-          <t>ELECTRICIDAD</t>
+          <t>MAESTRANZA</t>
         </is>
       </c>
       <c r="F88" s="6" t="inlineStr">
@@ -9973,17 +9985,17 @@
     <row r="89" ht="20" customHeight="1">
       <c r="A89" s="4" t="inlineStr">
         <is>
-          <t>71715827</t>
+          <t>70639427</t>
         </is>
       </c>
       <c r="B89" s="5" t="inlineStr">
         <is>
-          <t>ROJAS CASTRO</t>
+          <t>RUBIO GUTIERRES</t>
         </is>
       </c>
       <c r="C89" s="5" t="inlineStr">
         <is>
-          <t>ALAN JANDY</t>
+          <t>OSBERTO</t>
         </is>
       </c>
       <c r="D89" s="5" t="inlineStr">
@@ -9993,7 +10005,7 @@
       </c>
       <c r="E89" s="5" t="inlineStr">
         <is>
-          <t>MAESTRANZA</t>
+          <t>OPERACIONES</t>
         </is>
       </c>
       <c r="F89" s="6" t="inlineStr">
@@ -10070,17 +10082,17 @@
     <row r="90" ht="20" customHeight="1">
       <c r="A90" s="4" t="inlineStr">
         <is>
-          <t>70639427</t>
+          <t>44375240</t>
         </is>
       </c>
       <c r="B90" s="5" t="inlineStr">
         <is>
-          <t>RUBIO GUTIERRES</t>
+          <t>SANCHEZ PEREZ</t>
         </is>
       </c>
       <c r="C90" s="5" t="inlineStr">
         <is>
-          <t>OSBERTO</t>
+          <t>EDIN FRANCO</t>
         </is>
       </c>
       <c r="D90" s="5" t="inlineStr">
@@ -10090,7 +10102,7 @@
       </c>
       <c r="E90" s="5" t="inlineStr">
         <is>
-          <t>OPERACIONES</t>
+          <t>MANTENIMIENTO</t>
         </is>
       </c>
       <c r="F90" s="6" t="inlineStr">
@@ -10167,17 +10179,17 @@
     <row r="91" ht="20" customHeight="1">
       <c r="A91" s="4" t="inlineStr">
         <is>
-          <t>44375240</t>
+          <t>43240513</t>
         </is>
       </c>
       <c r="B91" s="5" t="inlineStr">
         <is>
-          <t>SANCHEZ PEREZ</t>
+          <t>SANTOS AGUSTIN</t>
         </is>
       </c>
       <c r="C91" s="5" t="inlineStr">
         <is>
-          <t>EDIN FRANCO</t>
+          <t>JUAN DIEGO</t>
         </is>
       </c>
       <c r="D91" s="5" t="inlineStr">
@@ -10187,7 +10199,7 @@
       </c>
       <c r="E91" s="5" t="inlineStr">
         <is>
-          <t>MANTENIMIENTO</t>
+          <t>CONDUCTOR</t>
         </is>
       </c>
       <c r="F91" s="6" t="inlineStr">
@@ -10264,17 +10276,17 @@
     <row r="92" ht="20" customHeight="1">
       <c r="A92" s="4" t="inlineStr">
         <is>
-          <t>43240513</t>
+          <t>41090271</t>
         </is>
       </c>
       <c r="B92" s="5" t="inlineStr">
         <is>
-          <t>SANTOS AGUSTIN</t>
+          <t>SILVA CORDOVA</t>
         </is>
       </c>
       <c r="C92" s="5" t="inlineStr">
         <is>
-          <t>JUAN DIEGO</t>
+          <t>JUAN PABLO</t>
         </is>
       </c>
       <c r="D92" s="5" t="inlineStr">
@@ -10284,7 +10296,7 @@
       </c>
       <c r="E92" s="5" t="inlineStr">
         <is>
-          <t>CONDUCTOR</t>
+          <t>OPERACIONES</t>
         </is>
       </c>
       <c r="F92" s="6" t="inlineStr">
@@ -10361,17 +10373,17 @@
     <row r="93" ht="20" customHeight="1">
       <c r="A93" s="4" t="inlineStr">
         <is>
-          <t>41090271</t>
+          <t>75539351</t>
         </is>
       </c>
       <c r="B93" s="5" t="inlineStr">
         <is>
-          <t>SILVA CORDOVA</t>
+          <t>SOLANO GONZALES</t>
         </is>
       </c>
       <c r="C93" s="5" t="inlineStr">
         <is>
-          <t>JUAN PABLO</t>
+          <t>YERSON BRADI</t>
         </is>
       </c>
       <c r="D93" s="5" t="inlineStr">
@@ -10458,27 +10470,27 @@
     <row r="94" ht="20" customHeight="1">
       <c r="A94" s="4" t="inlineStr">
         <is>
-          <t>75539351</t>
+          <t>26696602</t>
         </is>
       </c>
       <c r="B94" s="5" t="inlineStr">
         <is>
-          <t>SOLANO GONZALES</t>
+          <t>SÁNCHEZ MONTOYA</t>
         </is>
       </c>
       <c r="C94" s="5" t="inlineStr">
         <is>
-          <t>YERSON BRADI</t>
+          <t>MANUEL YSIDORO</t>
         </is>
       </c>
       <c r="D94" s="5" t="inlineStr">
         <is>
-          <t>OPER&amp;MTTO</t>
+          <t>JEFATURA</t>
         </is>
       </c>
       <c r="E94" s="5" t="inlineStr">
         <is>
-          <t>OPERACIONES</t>
+          <t>SUPERINTENDENTE</t>
         </is>
       </c>
       <c r="F94" s="6" t="inlineStr">
@@ -10555,27 +10567,27 @@
     <row r="95" ht="20" customHeight="1">
       <c r="A95" s="4" t="inlineStr">
         <is>
-          <t>26696602</t>
+          <t>75295662</t>
         </is>
       </c>
       <c r="B95" s="5" t="inlineStr">
         <is>
-          <t>SÁNCHEZ MONTOYA</t>
+          <t>TIMANA NAVARRO</t>
         </is>
       </c>
       <c r="C95" s="5" t="inlineStr">
         <is>
-          <t>MANUEL YSIDORO</t>
+          <t>ANDERSON ALDAHIR</t>
         </is>
       </c>
       <c r="D95" s="5" t="inlineStr">
         <is>
-          <t>JEFATURA</t>
+          <t>OPER&amp;MTTO</t>
         </is>
       </c>
       <c r="E95" s="5" t="inlineStr">
         <is>
-          <t>SUPERINTENDENTE</t>
+          <t>OPERACIONES</t>
         </is>
       </c>
       <c r="F95" s="6" t="inlineStr">
@@ -10652,17 +10664,17 @@
     <row r="96" ht="20" customHeight="1">
       <c r="A96" s="4" t="inlineStr">
         <is>
-          <t>75295662</t>
+          <t>73485498</t>
         </is>
       </c>
       <c r="B96" s="5" t="inlineStr">
         <is>
-          <t>TIMANA NAVARRO</t>
+          <t>VEGA CASTILLO</t>
         </is>
       </c>
       <c r="C96" s="5" t="inlineStr">
         <is>
-          <t>ANDERSON ALDAHIR</t>
+          <t>WILLY LEONARDO</t>
         </is>
       </c>
       <c r="D96" s="5" t="inlineStr">
@@ -10749,17 +10761,17 @@
     <row r="97" ht="20" customHeight="1">
       <c r="A97" s="4" t="inlineStr">
         <is>
-          <t>73485498</t>
+          <t>70480441</t>
         </is>
       </c>
       <c r="B97" s="5" t="inlineStr">
         <is>
-          <t>VEGA CASTILLO</t>
+          <t>CRUZ HUAMAN</t>
         </is>
       </c>
       <c r="C97" s="5" t="inlineStr">
         <is>
-          <t>WILLY LEONARDO</t>
+          <t>BRYAN ERNEST</t>
         </is>
       </c>
       <c r="D97" s="5" t="inlineStr">
@@ -10774,12 +10786,12 @@
       </c>
       <c r="F97" s="6" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="G97" s="6" t="inlineStr">
         <is>
-          <t>Lunes</t>
+          <t>Martes</t>
         </is>
       </c>
       <c r="H97" s="6" t="inlineStr">
@@ -10846,27 +10858,27 @@
     <row r="98" ht="20" customHeight="1">
       <c r="A98" s="4" t="inlineStr">
         <is>
-          <t>70480441</t>
+          <t>72559194</t>
         </is>
       </c>
       <c r="B98" s="5" t="inlineStr">
         <is>
-          <t>CRUZ HUAMAN</t>
+          <t>DE LA RIVA AGUILAR</t>
         </is>
       </c>
       <c r="C98" s="5" t="inlineStr">
         <is>
-          <t>BRYAN ERNEST</t>
+          <t>JAVIER ADRIAN</t>
         </is>
       </c>
       <c r="D98" s="5" t="inlineStr">
         <is>
-          <t>OPER&amp;MTTO</t>
+          <t>JEFATURA</t>
         </is>
       </c>
       <c r="E98" s="5" t="inlineStr">
         <is>
-          <t>OPERACIONES</t>
+          <t>SUPERVISOR</t>
         </is>
       </c>
       <c r="F98" s="6" t="inlineStr">
@@ -10943,27 +10955,27 @@
     <row r="99" ht="20" customHeight="1">
       <c r="A99" s="4" t="inlineStr">
         <is>
-          <t>72559194</t>
+          <t>46671923</t>
         </is>
       </c>
       <c r="B99" s="5" t="inlineStr">
         <is>
-          <t>DE LA RIVA AGUILAR</t>
+          <t>HUAYAMA ADRIANO</t>
         </is>
       </c>
       <c r="C99" s="5" t="inlineStr">
         <is>
-          <t>JAVIER ADRIAN</t>
+          <t>JOSMELL WALDIR</t>
         </is>
       </c>
       <c r="D99" s="5" t="inlineStr">
         <is>
-          <t>JEFATURA</t>
+          <t>OPER&amp;MTTO</t>
         </is>
       </c>
       <c r="E99" s="5" t="inlineStr">
         <is>
-          <t>SUPERVISOR</t>
+          <t>MANTENIMIENTO</t>
         </is>
       </c>
       <c r="F99" s="6" t="inlineStr">
@@ -11040,17 +11052,17 @@
     <row r="100" ht="20" customHeight="1">
       <c r="A100" s="4" t="inlineStr">
         <is>
-          <t>46671923</t>
+          <t>78378144</t>
         </is>
       </c>
       <c r="B100" s="5" t="inlineStr">
         <is>
-          <t>HUAYAMA ADRIANO</t>
+          <t>LADINES AGURTO</t>
         </is>
       </c>
       <c r="C100" s="5" t="inlineStr">
         <is>
-          <t>JOSMELL WALDIR</t>
+          <t>CRISTHIAN SINCLAIR</t>
         </is>
       </c>
       <c r="D100" s="5" t="inlineStr">
@@ -11060,7 +11072,7 @@
       </c>
       <c r="E100" s="5" t="inlineStr">
         <is>
-          <t>MANTENIMIENTO</t>
+          <t>MAESTRANZA</t>
         </is>
       </c>
       <c r="F100" s="6" t="inlineStr">
@@ -11137,7 +11149,7 @@
     <row r="101" ht="20" customHeight="1">
       <c r="A101" s="4" t="inlineStr">
         <is>
-          <t>78378144</t>
+          <t>62772089</t>
         </is>
       </c>
       <c r="B101" s="5" t="inlineStr">
@@ -11147,7 +11159,7 @@
       </c>
       <c r="C101" s="5" t="inlineStr">
         <is>
-          <t>CRISTHIAN SINCLAIR</t>
+          <t>JESUS GABRIEL</t>
         </is>
       </c>
       <c r="D101" s="5" t="inlineStr">
@@ -11157,7 +11169,7 @@
       </c>
       <c r="E101" s="5" t="inlineStr">
         <is>
-          <t>MAESTRANZA</t>
+          <t>OPERACIONES</t>
         </is>
       </c>
       <c r="F101" s="6" t="inlineStr">
@@ -11234,17 +11246,17 @@
     <row r="102" ht="20" customHeight="1">
       <c r="A102" s="4" t="inlineStr">
         <is>
-          <t>62772089</t>
+          <t>19571505</t>
         </is>
       </c>
       <c r="B102" s="5" t="inlineStr">
         <is>
-          <t>LADINES AGURTO</t>
+          <t>MARQUINA RIOS</t>
         </is>
       </c>
       <c r="C102" s="5" t="inlineStr">
         <is>
-          <t>JESUS GABRIEL</t>
+          <t>EDWARD GIOVANNY</t>
         </is>
       </c>
       <c r="D102" s="5" t="inlineStr">
@@ -11254,7 +11266,7 @@
       </c>
       <c r="E102" s="5" t="inlineStr">
         <is>
-          <t>OPERACIONES</t>
+          <t>MAESTRANZA</t>
         </is>
       </c>
       <c r="F102" s="6" t="inlineStr">
@@ -11331,17 +11343,17 @@
     <row r="103" ht="20" customHeight="1">
       <c r="A103" s="4" t="inlineStr">
         <is>
-          <t>19571505</t>
+          <t>19678776</t>
         </is>
       </c>
       <c r="B103" s="5" t="inlineStr">
         <is>
-          <t>MARQUINA RIOS</t>
+          <t>MAXIMILIANO CHACON</t>
         </is>
       </c>
       <c r="C103" s="5" t="inlineStr">
         <is>
-          <t>EDWARD GIOVANNY</t>
+          <t>SEBASTIAN</t>
         </is>
       </c>
       <c r="D103" s="5" t="inlineStr">
@@ -11351,7 +11363,7 @@
       </c>
       <c r="E103" s="5" t="inlineStr">
         <is>
-          <t>MAESTRANZA</t>
+          <t>OPERACIONES</t>
         </is>
       </c>
       <c r="F103" s="6" t="inlineStr">
@@ -11428,17 +11440,17 @@
     <row r="104" ht="20" customHeight="1">
       <c r="A104" s="4" t="inlineStr">
         <is>
-          <t>19678776</t>
+          <t>71715827</t>
         </is>
       </c>
       <c r="B104" s="5" t="inlineStr">
         <is>
-          <t>MAXIMILIANO CHACON</t>
+          <t>ROJAS CASTRO</t>
         </is>
       </c>
       <c r="C104" s="5" t="inlineStr">
         <is>
-          <t>SEBASTIAN</t>
+          <t>ALAN JANDY</t>
         </is>
       </c>
       <c r="D104" s="5" t="inlineStr">
@@ -11448,7 +11460,7 @@
       </c>
       <c r="E104" s="5" t="inlineStr">
         <is>
-          <t>OPERACIONES</t>
+          <t>MAESTRANZA</t>
         </is>
       </c>
       <c r="F104" s="6" t="inlineStr">
@@ -11525,17 +11537,17 @@
     <row r="105" ht="20" customHeight="1">
       <c r="A105" s="4" t="inlineStr">
         <is>
-          <t>03208053</t>
+          <t>70639427</t>
         </is>
       </c>
       <c r="B105" s="5" t="inlineStr">
         <is>
-          <t>MORETO BERMEO</t>
+          <t>RUBIO GUTIERRES</t>
         </is>
       </c>
       <c r="C105" s="5" t="inlineStr">
         <is>
-          <t>FRANCO</t>
+          <t>OSBERTO</t>
         </is>
       </c>
       <c r="D105" s="5" t="inlineStr">
@@ -11545,7 +11557,7 @@
       </c>
       <c r="E105" s="5" t="inlineStr">
         <is>
-          <t>MANTENIMIENTO</t>
+          <t>OPERACIONES</t>
         </is>
       </c>
       <c r="F105" s="6" t="inlineStr">
@@ -11622,17 +11634,17 @@
     <row r="106" ht="20" customHeight="1">
       <c r="A106" s="4" t="inlineStr">
         <is>
-          <t>006616501</t>
+          <t>44375240</t>
         </is>
       </c>
       <c r="B106" s="5" t="inlineStr">
         <is>
-          <t>ORDOÑEZ ARTEAGA</t>
+          <t>SANCHEZ PEREZ</t>
         </is>
       </c>
       <c r="C106" s="5" t="inlineStr">
         <is>
-          <t>YENKLI VICENTE</t>
+          <t>EDIN FRANCO</t>
         </is>
       </c>
       <c r="D106" s="5" t="inlineStr">
@@ -11642,7 +11654,7 @@
       </c>
       <c r="E106" s="5" t="inlineStr">
         <is>
-          <t>ELECTRICIDAD</t>
+          <t>MANTENIMIENTO</t>
         </is>
       </c>
       <c r="F106" s="6" t="inlineStr">
@@ -11719,17 +11731,17 @@
     <row r="107" ht="20" customHeight="1">
       <c r="A107" s="4" t="inlineStr">
         <is>
-          <t>71715827</t>
+          <t>43240513</t>
         </is>
       </c>
       <c r="B107" s="5" t="inlineStr">
         <is>
-          <t>ROJAS CASTRO</t>
+          <t>SANTOS AGUSTIN</t>
         </is>
       </c>
       <c r="C107" s="5" t="inlineStr">
         <is>
-          <t>ALAN JANDY</t>
+          <t>JUAN DIEGO</t>
         </is>
       </c>
       <c r="D107" s="5" t="inlineStr">
@@ -11739,7 +11751,7 @@
       </c>
       <c r="E107" s="5" t="inlineStr">
         <is>
-          <t>MAESTRANZA</t>
+          <t>CONDUCTOR</t>
         </is>
       </c>
       <c r="F107" s="6" t="inlineStr">
@@ -11816,17 +11828,17 @@
     <row r="108" ht="20" customHeight="1">
       <c r="A108" s="4" t="inlineStr">
         <is>
-          <t>70639427</t>
+          <t>41090271</t>
         </is>
       </c>
       <c r="B108" s="5" t="inlineStr">
         <is>
-          <t>RUBIO GUTIERRES</t>
+          <t>SILVA CORDOVA</t>
         </is>
       </c>
       <c r="C108" s="5" t="inlineStr">
         <is>
-          <t>OSBERTO</t>
+          <t>JUAN PABLO</t>
         </is>
       </c>
       <c r="D108" s="5" t="inlineStr">
@@ -11913,17 +11925,17 @@
     <row r="109" ht="20" customHeight="1">
       <c r="A109" s="4" t="inlineStr">
         <is>
-          <t>44375240</t>
+          <t>75539351</t>
         </is>
       </c>
       <c r="B109" s="5" t="inlineStr">
         <is>
-          <t>SANCHEZ PEREZ</t>
+          <t>SOLANO GONZALES</t>
         </is>
       </c>
       <c r="C109" s="5" t="inlineStr">
         <is>
-          <t>EDIN FRANCO</t>
+          <t>YERSON BRADI</t>
         </is>
       </c>
       <c r="D109" s="5" t="inlineStr">
@@ -11933,7 +11945,7 @@
       </c>
       <c r="E109" s="5" t="inlineStr">
         <is>
-          <t>MANTENIMIENTO</t>
+          <t>OPERACIONES</t>
         </is>
       </c>
       <c r="F109" s="6" t="inlineStr">
@@ -12010,27 +12022,27 @@
     <row r="110" ht="20" customHeight="1">
       <c r="A110" s="4" t="inlineStr">
         <is>
-          <t>43240513</t>
+          <t>26696602</t>
         </is>
       </c>
       <c r="B110" s="5" t="inlineStr">
         <is>
-          <t>SANTOS AGUSTIN</t>
+          <t>SÁNCHEZ MONTOYA</t>
         </is>
       </c>
       <c r="C110" s="5" t="inlineStr">
         <is>
-          <t>JUAN DIEGO</t>
+          <t>MANUEL YSIDORO</t>
         </is>
       </c>
       <c r="D110" s="5" t="inlineStr">
         <is>
-          <t>OPER&amp;MTTO</t>
+          <t>JEFATURA</t>
         </is>
       </c>
       <c r="E110" s="5" t="inlineStr">
         <is>
-          <t>CONDUCTOR</t>
+          <t>SUPERINTENDENTE</t>
         </is>
       </c>
       <c r="F110" s="6" t="inlineStr">
@@ -12107,17 +12119,17 @@
     <row r="111" ht="20" customHeight="1">
       <c r="A111" s="4" t="inlineStr">
         <is>
-          <t>41090271</t>
+          <t>75295662</t>
         </is>
       </c>
       <c r="B111" s="5" t="inlineStr">
         <is>
-          <t>SILVA CORDOVA</t>
+          <t>TIMANA NAVARRO</t>
         </is>
       </c>
       <c r="C111" s="5" t="inlineStr">
         <is>
-          <t>JUAN PABLO</t>
+          <t>ANDERSON ALDAHIR</t>
         </is>
       </c>
       <c r="D111" s="5" t="inlineStr">
@@ -12204,17 +12216,17 @@
     <row r="112" ht="20" customHeight="1">
       <c r="A112" s="4" t="inlineStr">
         <is>
-          <t>75539351</t>
+          <t>73485498</t>
         </is>
       </c>
       <c r="B112" s="5" t="inlineStr">
         <is>
-          <t>SOLANO GONZALES</t>
+          <t>VEGA CASTILLO</t>
         </is>
       </c>
       <c r="C112" s="5" t="inlineStr">
         <is>
-          <t>YERSON BRADI</t>
+          <t>WILLY LEONARDO</t>
         </is>
       </c>
       <c r="D112" s="5" t="inlineStr">
@@ -12297,297 +12309,6 @@
         </is>
       </c>
       <c r="W112" s="5" t="inlineStr"/>
-    </row>
-    <row r="113" ht="20" customHeight="1">
-      <c r="A113" s="4" t="inlineStr">
-        <is>
-          <t>26696602</t>
-        </is>
-      </c>
-      <c r="B113" s="5" t="inlineStr">
-        <is>
-          <t>SÁNCHEZ MONTOYA</t>
-        </is>
-      </c>
-      <c r="C113" s="5" t="inlineStr">
-        <is>
-          <t>MANUEL YSIDORO</t>
-        </is>
-      </c>
-      <c r="D113" s="5" t="inlineStr">
-        <is>
-          <t>JEFATURA</t>
-        </is>
-      </c>
-      <c r="E113" s="5" t="inlineStr">
-        <is>
-          <t>SUPERINTENDENTE</t>
-        </is>
-      </c>
-      <c r="F113" s="6" t="inlineStr">
-        <is>
-          <t>2026-08-18</t>
-        </is>
-      </c>
-      <c r="G113" s="6" t="inlineStr">
-        <is>
-          <t>Martes</t>
-        </is>
-      </c>
-      <c r="H113" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="I113" s="6" t="inlineStr"/>
-      <c r="J113" s="6" t="inlineStr"/>
-      <c r="K113" s="6" t="inlineStr"/>
-      <c r="L113" s="6" t="inlineStr"/>
-      <c r="M113" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N113" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O113" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P113" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q113" s="6" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="R113" s="6" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="S113" s="6" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="T113" s="6" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="U113" s="6" t="inlineStr">
-        <is>
-          <t>Huella dactilar</t>
-        </is>
-      </c>
-      <c r="V113" s="6" t="inlineStr">
-        <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="W113" s="5" t="inlineStr"/>
-    </row>
-    <row r="114" ht="20" customHeight="1">
-      <c r="A114" s="4" t="inlineStr">
-        <is>
-          <t>75295662</t>
-        </is>
-      </c>
-      <c r="B114" s="5" t="inlineStr">
-        <is>
-          <t>TIMANA NAVARRO</t>
-        </is>
-      </c>
-      <c r="C114" s="5" t="inlineStr">
-        <is>
-          <t>ANDERSON ALDAHIR</t>
-        </is>
-      </c>
-      <c r="D114" s="5" t="inlineStr">
-        <is>
-          <t>OPER&amp;MTTO</t>
-        </is>
-      </c>
-      <c r="E114" s="5" t="inlineStr">
-        <is>
-          <t>OPERACIONES</t>
-        </is>
-      </c>
-      <c r="F114" s="6" t="inlineStr">
-        <is>
-          <t>2026-08-18</t>
-        </is>
-      </c>
-      <c r="G114" s="6" t="inlineStr">
-        <is>
-          <t>Martes</t>
-        </is>
-      </c>
-      <c r="H114" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="I114" s="6" t="inlineStr"/>
-      <c r="J114" s="6" t="inlineStr"/>
-      <c r="K114" s="6" t="inlineStr"/>
-      <c r="L114" s="6" t="inlineStr"/>
-      <c r="M114" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N114" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O114" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P114" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q114" s="6" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="R114" s="6" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="S114" s="6" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="T114" s="6" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="U114" s="6" t="inlineStr">
-        <is>
-          <t>Huella dactilar</t>
-        </is>
-      </c>
-      <c r="V114" s="6" t="inlineStr">
-        <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="W114" s="5" t="inlineStr"/>
-    </row>
-    <row r="115" ht="20" customHeight="1">
-      <c r="A115" s="4" t="inlineStr">
-        <is>
-          <t>73485498</t>
-        </is>
-      </c>
-      <c r="B115" s="5" t="inlineStr">
-        <is>
-          <t>VEGA CASTILLO</t>
-        </is>
-      </c>
-      <c r="C115" s="5" t="inlineStr">
-        <is>
-          <t>WILLY LEONARDO</t>
-        </is>
-      </c>
-      <c r="D115" s="5" t="inlineStr">
-        <is>
-          <t>OPER&amp;MTTO</t>
-        </is>
-      </c>
-      <c r="E115" s="5" t="inlineStr">
-        <is>
-          <t>OPERACIONES</t>
-        </is>
-      </c>
-      <c r="F115" s="6" t="inlineStr">
-        <is>
-          <t>2026-08-18</t>
-        </is>
-      </c>
-      <c r="G115" s="6" t="inlineStr">
-        <is>
-          <t>Martes</t>
-        </is>
-      </c>
-      <c r="H115" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="I115" s="6" t="inlineStr"/>
-      <c r="J115" s="6" t="inlineStr"/>
-      <c r="K115" s="6" t="inlineStr"/>
-      <c r="L115" s="6" t="inlineStr"/>
-      <c r="M115" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N115" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O115" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P115" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q115" s="6" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="R115" s="6" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="S115" s="6" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="T115" s="6" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="U115" s="6" t="inlineStr">
-        <is>
-          <t>Huella dactilar</t>
-        </is>
-      </c>
-      <c r="V115" s="6" t="inlineStr">
-        <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="W115" s="5" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
Fix Turno Noche cross-date pairing for evening entries and morning exits (e.g. Sangabil Guerra Sajami)
</commit_message>
<xml_diff>
--- a/Sistema_Asistencia_GZG_v1.0.xlsx
+++ b/Sistema_Asistencia_GZG_v1.0.xlsx
@@ -1726,7 +1726,11 @@
           <t>06:46</t>
         </is>
       </c>
-      <c r="K14" s="6" t="inlineStr"/>
+      <c r="K14" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
       <c r="L14" s="6" t="inlineStr"/>
       <c r="M14" s="6" t="inlineStr">
         <is>
@@ -1948,8 +1952,16 @@
           <t>18:16</t>
         </is>
       </c>
-      <c r="K16" s="6" t="inlineStr"/>
-      <c r="L16" s="6" t="inlineStr"/>
+      <c r="K16" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="L16" s="6" t="inlineStr">
+        <is>
+          <t>07:01</t>
+        </is>
+      </c>
       <c r="M16" s="6" t="inlineStr">
         <is>
           <t>-</t>
@@ -1972,7 +1984,7 @@
       </c>
       <c r="Q16" s="6" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>12:45</t>
         </is>
       </c>
       <c r="R16" s="6" t="inlineStr">
@@ -1982,12 +1994,12 @@
       </c>
       <c r="S16" s="6" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>00:01</t>
         </is>
       </c>
       <c r="T16" s="6" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>00:01</t>
         </is>
       </c>
       <c r="U16" s="6" t="inlineStr">
@@ -2044,21 +2056,21 @@
       </c>
       <c r="H17" s="6" t="inlineStr">
         <is>
-          <t>NOCHE</t>
-        </is>
-      </c>
-      <c r="I17" s="6" t="inlineStr"/>
+          <t>DIA</t>
+        </is>
+      </c>
+      <c r="I17" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
       <c r="J17" s="6" t="inlineStr"/>
       <c r="K17" s="6" t="inlineStr">
         <is>
           <t>2026-08-18</t>
         </is>
       </c>
-      <c r="L17" s="6" t="inlineStr">
-        <is>
-          <t>07:01</t>
-        </is>
-      </c>
+      <c r="L17" s="6" t="inlineStr"/>
       <c r="M17" s="6" t="inlineStr">
         <is>
           <t>-</t>
@@ -2106,14 +2118,10 @@
       </c>
       <c r="V17" s="6" t="inlineStr">
         <is>
-          <t>Salida sin entrada</t>
-        </is>
-      </c>
-      <c r="W17" s="5" t="inlineStr">
-        <is>
-          <t>Salida sin registro de entrada previa (07:01)</t>
-        </is>
-      </c>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="W17" s="5" t="inlineStr"/>
     </row>
     <row r="18" ht="20" customHeight="1">
       <c r="A18" s="4" t="inlineStr">
@@ -3877,7 +3885,11 @@
           <t>07:20</t>
         </is>
       </c>
-      <c r="K33" s="6" t="inlineStr"/>
+      <c r="K33" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
       <c r="L33" s="6" t="inlineStr"/>
       <c r="M33" s="6" t="inlineStr">
         <is>
@@ -4103,8 +4115,16 @@
           <t>18:50</t>
         </is>
       </c>
-      <c r="K35" s="6" t="inlineStr"/>
-      <c r="L35" s="6" t="inlineStr"/>
+      <c r="K35" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="L35" s="6" t="inlineStr">
+        <is>
+          <t>07:01</t>
+        </is>
+      </c>
       <c r="M35" s="6" t="inlineStr">
         <is>
           <t>-</t>
@@ -4127,7 +4147,7 @@
       </c>
       <c r="Q35" s="6" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>12:11</t>
         </is>
       </c>
       <c r="R35" s="6" t="inlineStr">
@@ -4137,12 +4157,12 @@
       </c>
       <c r="S35" s="6" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>00:01</t>
         </is>
       </c>
       <c r="T35" s="6" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>00:01</t>
         </is>
       </c>
       <c r="U35" s="6" t="inlineStr">
@@ -4155,11 +4175,7 @@
           <t>Normal</t>
         </is>
       </c>
-      <c r="W35" s="5" t="inlineStr">
-        <is>
-          <t>Falta marcación de salida</t>
-        </is>
-      </c>
+      <c r="W35" s="5" t="inlineStr"/>
     </row>
     <row r="36" ht="20" customHeight="1">
       <c r="A36" s="4" t="inlineStr">
@@ -4217,11 +4233,7 @@
           <t>2026-08-18</t>
         </is>
       </c>
-      <c r="L36" s="6" t="inlineStr">
-        <is>
-          <t>07:01</t>
-        </is>
-      </c>
+      <c r="L36" s="6" t="inlineStr"/>
       <c r="M36" s="6" t="inlineStr">
         <is>
           <t>-</t>
@@ -4244,7 +4256,7 @@
       </c>
       <c r="Q36" s="6" t="inlineStr">
         <is>
-          <t>12:21</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="R36" s="6" t="inlineStr">
@@ -4254,12 +4266,12 @@
       </c>
       <c r="S36" s="6" t="inlineStr">
         <is>
-          <t>00:01</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="T36" s="6" t="inlineStr">
         <is>
-          <t>00:01</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="U36" s="6" t="inlineStr">
@@ -4272,7 +4284,11 @@
           <t>Normal</t>
         </is>
       </c>
-      <c r="W36" s="5" t="inlineStr"/>
+      <c r="W36" s="5" t="inlineStr">
+        <is>
+          <t>Falta marcación de salida</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="20" customHeight="1">
       <c r="A37" s="4" t="inlineStr">
@@ -4559,8 +4575,16 @@
           <t>18:32</t>
         </is>
       </c>
-      <c r="K39" s="6" t="inlineStr"/>
-      <c r="L39" s="6" t="inlineStr"/>
+      <c r="K39" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="L39" s="6" t="inlineStr">
+        <is>
+          <t>07:01</t>
+        </is>
+      </c>
       <c r="M39" s="6" t="inlineStr">
         <is>
           <t>-</t>
@@ -4583,7 +4607,7 @@
       </c>
       <c r="Q39" s="6" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>12:29</t>
         </is>
       </c>
       <c r="R39" s="6" t="inlineStr">
@@ -4593,12 +4617,12 @@
       </c>
       <c r="S39" s="6" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>00:01</t>
         </is>
       </c>
       <c r="T39" s="6" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>00:01</t>
         </is>
       </c>
       <c r="U39" s="6" t="inlineStr">
@@ -4611,11 +4635,7 @@
           <t>Normal</t>
         </is>
       </c>
-      <c r="W39" s="5" t="inlineStr">
-        <is>
-          <t>Falta marcación de salida</t>
-        </is>
-      </c>
+      <c r="W39" s="5" t="inlineStr"/>
     </row>
     <row r="40" ht="20" customHeight="1">
       <c r="A40" s="4" t="inlineStr">
@@ -4673,11 +4693,7 @@
           <t>2026-08-18</t>
         </is>
       </c>
-      <c r="L40" s="6" t="inlineStr">
-        <is>
-          <t>07:01</t>
-        </is>
-      </c>
+      <c r="L40" s="6" t="inlineStr"/>
       <c r="M40" s="6" t="inlineStr">
         <is>
           <t>-</t>
@@ -4700,7 +4716,7 @@
       </c>
       <c r="Q40" s="6" t="inlineStr">
         <is>
-          <t>12:30</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="R40" s="6" t="inlineStr">
@@ -4710,12 +4726,12 @@
       </c>
       <c r="S40" s="6" t="inlineStr">
         <is>
-          <t>00:01</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="T40" s="6" t="inlineStr">
         <is>
-          <t>00:01</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="U40" s="6" t="inlineStr">
@@ -4728,7 +4744,11 @@
           <t>Normal</t>
         </is>
       </c>
-      <c r="W40" s="5" t="inlineStr"/>
+      <c r="W40" s="5" t="inlineStr">
+        <is>
+          <t>Falta marcación de salida</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="20" customHeight="1">
       <c r="A41" s="4" t="inlineStr">
@@ -4781,8 +4801,16 @@
           <t>19:56</t>
         </is>
       </c>
-      <c r="K41" s="6" t="inlineStr"/>
-      <c r="L41" s="6" t="inlineStr"/>
+      <c r="K41" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="L41" s="6" t="inlineStr">
+        <is>
+          <t>07:06</t>
+        </is>
+      </c>
       <c r="M41" s="6" t="inlineStr">
         <is>
           <t>-</t>
@@ -4805,7 +4833,7 @@
       </c>
       <c r="Q41" s="6" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>11:10</t>
         </is>
       </c>
       <c r="R41" s="6" t="inlineStr">
@@ -4815,12 +4843,12 @@
       </c>
       <c r="S41" s="6" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>00:06</t>
         </is>
       </c>
       <c r="T41" s="6" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>00:06</t>
         </is>
       </c>
       <c r="U41" s="6" t="inlineStr">
@@ -4835,7 +4863,7 @@
       </c>
       <c r="W41" s="5" t="inlineStr">
         <is>
-          <t>Falta marcación de salida, Tardanza (41 min)</t>
+          <t>Tardanza (41 min)</t>
         </is>
       </c>
     </row>
@@ -4895,11 +4923,7 @@
           <t>2026-08-18</t>
         </is>
       </c>
-      <c r="L42" s="6" t="inlineStr">
-        <is>
-          <t>07:06</t>
-        </is>
-      </c>
+      <c r="L42" s="6" t="inlineStr"/>
       <c r="M42" s="6" t="inlineStr">
         <is>
           <t>-</t>
@@ -4922,7 +4946,7 @@
       </c>
       <c r="Q42" s="6" t="inlineStr">
         <is>
-          <t>12:35</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="R42" s="6" t="inlineStr">
@@ -4932,12 +4956,12 @@
       </c>
       <c r="S42" s="6" t="inlineStr">
         <is>
-          <t>00:06</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="T42" s="6" t="inlineStr">
         <is>
-          <t>00:06</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="U42" s="6" t="inlineStr">
@@ -4950,7 +4974,11 @@
           <t>Normal</t>
         </is>
       </c>
-      <c r="W42" s="5" t="inlineStr"/>
+      <c r="W42" s="5" t="inlineStr">
+        <is>
+          <t>Falta marcación de salida</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="20" customHeight="1">
       <c r="A43" s="4" t="inlineStr">
@@ -5227,7 +5255,11 @@
           <t>DIA</t>
         </is>
       </c>
-      <c r="I45" s="6" t="inlineStr"/>
+      <c r="I45" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
       <c r="J45" s="6" t="inlineStr"/>
       <c r="K45" s="6" t="inlineStr">
         <is>
@@ -5459,8 +5491,16 @@
           <t>18:32</t>
         </is>
       </c>
-      <c r="K47" s="6" t="inlineStr"/>
-      <c r="L47" s="6" t="inlineStr"/>
+      <c r="K47" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="L47" s="6" t="inlineStr">
+        <is>
+          <t>07:00</t>
+        </is>
+      </c>
       <c r="M47" s="6" t="inlineStr">
         <is>
           <t>-</t>
@@ -5483,7 +5523,7 @@
       </c>
       <c r="Q47" s="6" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>12:28</t>
         </is>
       </c>
       <c r="R47" s="6" t="inlineStr">
@@ -5511,11 +5551,7 @@
           <t>Normal</t>
         </is>
       </c>
-      <c r="W47" s="5" t="inlineStr">
-        <is>
-          <t>Falta marcación de salida</t>
-        </is>
-      </c>
+      <c r="W47" s="5" t="inlineStr"/>
     </row>
     <row r="48" ht="20" customHeight="1">
       <c r="A48" s="4" t="inlineStr">
@@ -5573,11 +5609,7 @@
           <t>2026-08-18</t>
         </is>
       </c>
-      <c r="L48" s="6" t="inlineStr">
-        <is>
-          <t>07:00</t>
-        </is>
-      </c>
+      <c r="L48" s="6" t="inlineStr"/>
       <c r="M48" s="6" t="inlineStr">
         <is>
           <t>-</t>
@@ -5600,7 +5632,7 @@
       </c>
       <c r="Q48" s="6" t="inlineStr">
         <is>
-          <t>12:31</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="R48" s="6" t="inlineStr">
@@ -5628,7 +5660,11 @@
           <t>Normal</t>
         </is>
       </c>
-      <c r="W48" s="5" t="inlineStr"/>
+      <c r="W48" s="5" t="inlineStr">
+        <is>
+          <t>Falta marcación de salida</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="20" customHeight="1">
       <c r="A49" s="4" t="inlineStr">
@@ -5681,8 +5717,16 @@
           <t>18:32</t>
         </is>
       </c>
-      <c r="K49" s="6" t="inlineStr"/>
-      <c r="L49" s="6" t="inlineStr"/>
+      <c r="K49" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="L49" s="6" t="inlineStr">
+        <is>
+          <t>07:00</t>
+        </is>
+      </c>
       <c r="M49" s="6" t="inlineStr">
         <is>
           <t>-</t>
@@ -5705,7 +5749,7 @@
       </c>
       <c r="Q49" s="6" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>12:28</t>
         </is>
       </c>
       <c r="R49" s="6" t="inlineStr">
@@ -5733,11 +5777,7 @@
           <t>Normal</t>
         </is>
       </c>
-      <c r="W49" s="5" t="inlineStr">
-        <is>
-          <t>Falta marcación de salida</t>
-        </is>
-      </c>
+      <c r="W49" s="5" t="inlineStr"/>
     </row>
     <row r="50" ht="20" customHeight="1">
       <c r="A50" s="4" t="inlineStr">
@@ -5795,11 +5835,7 @@
           <t>2026-08-18</t>
         </is>
       </c>
-      <c r="L50" s="6" t="inlineStr">
-        <is>
-          <t>07:00</t>
-        </is>
-      </c>
+      <c r="L50" s="6" t="inlineStr"/>
       <c r="M50" s="6" t="inlineStr">
         <is>
           <t>-</t>
@@ -5822,7 +5858,7 @@
       </c>
       <c r="Q50" s="6" t="inlineStr">
         <is>
-          <t>12:31</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="R50" s="6" t="inlineStr">
@@ -5850,7 +5886,11 @@
           <t>Normal</t>
         </is>
       </c>
-      <c r="W50" s="5" t="inlineStr"/>
+      <c r="W50" s="5" t="inlineStr">
+        <is>
+          <t>Falta marcación de salida</t>
+        </is>
+      </c>
     </row>
     <row r="51" ht="20" customHeight="1">
       <c r="A51" s="4" t="inlineStr">
@@ -5903,8 +5943,16 @@
           <t>18:38</t>
         </is>
       </c>
-      <c r="K51" s="6" t="inlineStr"/>
-      <c r="L51" s="6" t="inlineStr"/>
+      <c r="K51" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="L51" s="6" t="inlineStr">
+        <is>
+          <t>06:55</t>
+        </is>
+      </c>
       <c r="M51" s="6" t="inlineStr">
         <is>
           <t>-</t>
@@ -5927,7 +5975,7 @@
       </c>
       <c r="Q51" s="6" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>12:17</t>
         </is>
       </c>
       <c r="R51" s="6" t="inlineStr">
@@ -5955,11 +6003,7 @@
           <t>Normal</t>
         </is>
       </c>
-      <c r="W51" s="5" t="inlineStr">
-        <is>
-          <t>Falta marcación de salida</t>
-        </is>
-      </c>
+      <c r="W51" s="5" t="inlineStr"/>
     </row>
     <row r="52" ht="20" customHeight="1">
       <c r="A52" s="4" t="inlineStr">
@@ -6351,8 +6395,16 @@
           <t>18:38</t>
         </is>
       </c>
-      <c r="K55" s="6" t="inlineStr"/>
-      <c r="L55" s="6" t="inlineStr"/>
+      <c r="K55" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="L55" s="6" t="inlineStr">
+        <is>
+          <t>07:02</t>
+        </is>
+      </c>
       <c r="M55" s="6" t="inlineStr">
         <is>
           <t>-</t>
@@ -6375,7 +6427,7 @@
       </c>
       <c r="Q55" s="6" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>12:24</t>
         </is>
       </c>
       <c r="R55" s="6" t="inlineStr">
@@ -6385,12 +6437,12 @@
       </c>
       <c r="S55" s="6" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>00:02</t>
         </is>
       </c>
       <c r="T55" s="6" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>00:02</t>
         </is>
       </c>
       <c r="U55" s="6" t="inlineStr">
@@ -6403,11 +6455,7 @@
           <t>Normal</t>
         </is>
       </c>
-      <c r="W55" s="5" t="inlineStr">
-        <is>
-          <t>Falta marcación de salida</t>
-        </is>
-      </c>
+      <c r="W55" s="5" t="inlineStr"/>
     </row>
     <row r="56" ht="20" customHeight="1">
       <c r="A56" s="4" t="inlineStr">
@@ -6465,11 +6513,7 @@
           <t>2026-08-18</t>
         </is>
       </c>
-      <c r="L56" s="6" t="inlineStr">
-        <is>
-          <t>07:02</t>
-        </is>
-      </c>
+      <c r="L56" s="6" t="inlineStr"/>
       <c r="M56" s="6" t="inlineStr">
         <is>
           <t>-</t>
@@ -6492,7 +6536,7 @@
       </c>
       <c r="Q56" s="6" t="inlineStr">
         <is>
-          <t>12:27</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="R56" s="6" t="inlineStr">
@@ -6502,12 +6546,12 @@
       </c>
       <c r="S56" s="6" t="inlineStr">
         <is>
-          <t>00:02</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="T56" s="6" t="inlineStr">
         <is>
-          <t>00:02</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="U56" s="6" t="inlineStr">
@@ -6520,7 +6564,11 @@
           <t>Normal</t>
         </is>
       </c>
-      <c r="W56" s="5" t="inlineStr"/>
+      <c r="W56" s="5" t="inlineStr">
+        <is>
+          <t>Falta marcación de salida</t>
+        </is>
+      </c>
     </row>
     <row r="57" ht="20" customHeight="1">
       <c r="A57" s="4" t="inlineStr">
@@ -8619,8 +8667,16 @@
           <t>18:33</t>
         </is>
       </c>
-      <c r="K75" s="6" t="inlineStr"/>
-      <c r="L75" s="6" t="inlineStr"/>
+      <c r="K75" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="L75" s="6" t="inlineStr">
+        <is>
+          <t>07:00</t>
+        </is>
+      </c>
       <c r="M75" s="6" t="inlineStr">
         <is>
           <t>-</t>
@@ -8643,7 +8699,7 @@
       </c>
       <c r="Q75" s="6" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>12:27</t>
         </is>
       </c>
       <c r="R75" s="6" t="inlineStr">
@@ -8671,11 +8727,7 @@
           <t>Normal</t>
         </is>
       </c>
-      <c r="W75" s="5" t="inlineStr">
-        <is>
-          <t>Falta marcación de salida</t>
-        </is>
-      </c>
+      <c r="W75" s="5" t="inlineStr"/>
     </row>
     <row r="76" ht="20" customHeight="1">
       <c r="A76" s="4" t="inlineStr">
@@ -8733,11 +8785,7 @@
           <t>2026-08-18</t>
         </is>
       </c>
-      <c r="L76" s="6" t="inlineStr">
-        <is>
-          <t>07:00</t>
-        </is>
-      </c>
+      <c r="L76" s="6" t="inlineStr"/>
       <c r="M76" s="6" t="inlineStr">
         <is>
           <t>-</t>
@@ -8760,7 +8808,7 @@
       </c>
       <c r="Q76" s="6" t="inlineStr">
         <is>
-          <t>12:29</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="R76" s="6" t="inlineStr">
@@ -8788,7 +8836,11 @@
           <t>Normal</t>
         </is>
       </c>
-      <c r="W76" s="5" t="inlineStr"/>
+      <c r="W76" s="5" t="inlineStr">
+        <is>
+          <t>Falta marcación de salida</t>
+        </is>
+      </c>
     </row>
     <row r="77" ht="20" customHeight="1">
       <c r="A77" s="4" t="inlineStr">
@@ -8841,8 +8893,16 @@
           <t>18:37</t>
         </is>
       </c>
-      <c r="K77" s="6" t="inlineStr"/>
-      <c r="L77" s="6" t="inlineStr"/>
+      <c r="K77" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="L77" s="6" t="inlineStr">
+        <is>
+          <t>07:06</t>
+        </is>
+      </c>
       <c r="M77" s="6" t="inlineStr">
         <is>
           <t>-</t>
@@ -8865,7 +8925,7 @@
       </c>
       <c r="Q77" s="6" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>12:29</t>
         </is>
       </c>
       <c r="R77" s="6" t="inlineStr">
@@ -8875,12 +8935,12 @@
       </c>
       <c r="S77" s="6" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>00:06</t>
         </is>
       </c>
       <c r="T77" s="6" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>00:06</t>
         </is>
       </c>
       <c r="U77" s="6" t="inlineStr">
@@ -8893,11 +8953,7 @@
           <t>Normal</t>
         </is>
       </c>
-      <c r="W77" s="5" t="inlineStr">
-        <is>
-          <t>Falta marcación de salida</t>
-        </is>
-      </c>
+      <c r="W77" s="5" t="inlineStr"/>
     </row>
     <row r="78" ht="20" customHeight="1">
       <c r="A78" s="4" t="inlineStr">
@@ -8955,11 +9011,7 @@
           <t>2026-08-18</t>
         </is>
       </c>
-      <c r="L78" s="6" t="inlineStr">
-        <is>
-          <t>07:06</t>
-        </is>
-      </c>
+      <c r="L78" s="6" t="inlineStr"/>
       <c r="M78" s="6" t="inlineStr">
         <is>
           <t>-</t>
@@ -8982,7 +9034,7 @@
       </c>
       <c r="Q78" s="6" t="inlineStr">
         <is>
-          <t>12:35</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="R78" s="6" t="inlineStr">
@@ -8992,12 +9044,12 @@
       </c>
       <c r="S78" s="6" t="inlineStr">
         <is>
-          <t>00:06</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="T78" s="6" t="inlineStr">
         <is>
-          <t>00:06</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="U78" s="6" t="inlineStr">
@@ -9010,7 +9062,11 @@
           <t>Normal</t>
         </is>
       </c>
-      <c r="W78" s="5" t="inlineStr"/>
+      <c r="W78" s="5" t="inlineStr">
+        <is>
+          <t>Falta marcación de salida</t>
+        </is>
+      </c>
     </row>
     <row r="79" ht="20" customHeight="1">
       <c r="A79" s="4" t="inlineStr">
@@ -9053,9 +9109,17 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="I79" s="6" t="inlineStr"/>
+      <c r="I79" s="6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="J79" s="6" t="inlineStr"/>
-      <c r="K79" s="6" t="inlineStr"/>
+      <c r="K79" s="6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L79" s="6" t="inlineStr"/>
       <c r="M79" s="6" t="inlineStr">
         <is>
@@ -9150,9 +9214,17 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="I80" s="6" t="inlineStr"/>
+      <c r="I80" s="6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="J80" s="6" t="inlineStr"/>
-      <c r="K80" s="6" t="inlineStr"/>
+      <c r="K80" s="6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L80" s="6" t="inlineStr"/>
       <c r="M80" s="6" t="inlineStr">
         <is>
@@ -9247,9 +9319,17 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="I81" s="6" t="inlineStr"/>
+      <c r="I81" s="6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="J81" s="6" t="inlineStr"/>
-      <c r="K81" s="6" t="inlineStr"/>
+      <c r="K81" s="6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L81" s="6" t="inlineStr"/>
       <c r="M81" s="6" t="inlineStr">
         <is>
@@ -9344,9 +9424,17 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="I82" s="6" t="inlineStr"/>
+      <c r="I82" s="6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="J82" s="6" t="inlineStr"/>
-      <c r="K82" s="6" t="inlineStr"/>
+      <c r="K82" s="6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L82" s="6" t="inlineStr"/>
       <c r="M82" s="6" t="inlineStr">
         <is>
@@ -9441,9 +9529,17 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="I83" s="6" t="inlineStr"/>
+      <c r="I83" s="6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="J83" s="6" t="inlineStr"/>
-      <c r="K83" s="6" t="inlineStr"/>
+      <c r="K83" s="6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L83" s="6" t="inlineStr"/>
       <c r="M83" s="6" t="inlineStr">
         <is>
@@ -9538,9 +9634,17 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="I84" s="6" t="inlineStr"/>
+      <c r="I84" s="6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="J84" s="6" t="inlineStr"/>
-      <c r="K84" s="6" t="inlineStr"/>
+      <c r="K84" s="6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L84" s="6" t="inlineStr"/>
       <c r="M84" s="6" t="inlineStr">
         <is>
@@ -9635,9 +9739,17 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="I85" s="6" t="inlineStr"/>
+      <c r="I85" s="6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="J85" s="6" t="inlineStr"/>
-      <c r="K85" s="6" t="inlineStr"/>
+      <c r="K85" s="6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L85" s="6" t="inlineStr"/>
       <c r="M85" s="6" t="inlineStr">
         <is>
@@ -9732,9 +9844,17 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="I86" s="6" t="inlineStr"/>
+      <c r="I86" s="6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="J86" s="6" t="inlineStr"/>
-      <c r="K86" s="6" t="inlineStr"/>
+      <c r="K86" s="6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L86" s="6" t="inlineStr"/>
       <c r="M86" s="6" t="inlineStr">
         <is>
@@ -9829,9 +9949,17 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="I87" s="6" t="inlineStr"/>
+      <c r="I87" s="6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="J87" s="6" t="inlineStr"/>
-      <c r="K87" s="6" t="inlineStr"/>
+      <c r="K87" s="6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L87" s="6" t="inlineStr"/>
       <c r="M87" s="6" t="inlineStr">
         <is>
@@ -9926,9 +10054,17 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="I88" s="6" t="inlineStr"/>
+      <c r="I88" s="6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="J88" s="6" t="inlineStr"/>
-      <c r="K88" s="6" t="inlineStr"/>
+      <c r="K88" s="6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L88" s="6" t="inlineStr"/>
       <c r="M88" s="6" t="inlineStr">
         <is>
@@ -10023,9 +10159,17 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="I89" s="6" t="inlineStr"/>
+      <c r="I89" s="6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="J89" s="6" t="inlineStr"/>
-      <c r="K89" s="6" t="inlineStr"/>
+      <c r="K89" s="6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L89" s="6" t="inlineStr"/>
       <c r="M89" s="6" t="inlineStr">
         <is>
@@ -10120,9 +10264,17 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="I90" s="6" t="inlineStr"/>
+      <c r="I90" s="6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="J90" s="6" t="inlineStr"/>
-      <c r="K90" s="6" t="inlineStr"/>
+      <c r="K90" s="6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L90" s="6" t="inlineStr"/>
       <c r="M90" s="6" t="inlineStr">
         <is>
@@ -10217,9 +10369,17 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="I91" s="6" t="inlineStr"/>
+      <c r="I91" s="6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="J91" s="6" t="inlineStr"/>
-      <c r="K91" s="6" t="inlineStr"/>
+      <c r="K91" s="6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L91" s="6" t="inlineStr"/>
       <c r="M91" s="6" t="inlineStr">
         <is>
@@ -10314,9 +10474,17 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="I92" s="6" t="inlineStr"/>
+      <c r="I92" s="6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="J92" s="6" t="inlineStr"/>
-      <c r="K92" s="6" t="inlineStr"/>
+      <c r="K92" s="6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L92" s="6" t="inlineStr"/>
       <c r="M92" s="6" t="inlineStr">
         <is>
@@ -10411,9 +10579,17 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="I93" s="6" t="inlineStr"/>
+      <c r="I93" s="6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="J93" s="6" t="inlineStr"/>
-      <c r="K93" s="6" t="inlineStr"/>
+      <c r="K93" s="6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L93" s="6" t="inlineStr"/>
       <c r="M93" s="6" t="inlineStr">
         <is>
@@ -10508,9 +10684,17 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="I94" s="6" t="inlineStr"/>
+      <c r="I94" s="6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="J94" s="6" t="inlineStr"/>
-      <c r="K94" s="6" t="inlineStr"/>
+      <c r="K94" s="6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L94" s="6" t="inlineStr"/>
       <c r="M94" s="6" t="inlineStr">
         <is>
@@ -10605,9 +10789,17 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="I95" s="6" t="inlineStr"/>
+      <c r="I95" s="6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="J95" s="6" t="inlineStr"/>
-      <c r="K95" s="6" t="inlineStr"/>
+      <c r="K95" s="6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L95" s="6" t="inlineStr"/>
       <c r="M95" s="6" t="inlineStr">
         <is>
@@ -10702,9 +10894,17 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="I96" s="6" t="inlineStr"/>
+      <c r="I96" s="6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="J96" s="6" t="inlineStr"/>
-      <c r="K96" s="6" t="inlineStr"/>
+      <c r="K96" s="6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L96" s="6" t="inlineStr"/>
       <c r="M96" s="6" t="inlineStr">
         <is>
@@ -10799,9 +10999,17 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="I97" s="6" t="inlineStr"/>
+      <c r="I97" s="6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="J97" s="6" t="inlineStr"/>
-      <c r="K97" s="6" t="inlineStr"/>
+      <c r="K97" s="6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L97" s="6" t="inlineStr"/>
       <c r="M97" s="6" t="inlineStr">
         <is>
@@ -10896,9 +11104,17 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="I98" s="6" t="inlineStr"/>
+      <c r="I98" s="6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="J98" s="6" t="inlineStr"/>
-      <c r="K98" s="6" t="inlineStr"/>
+      <c r="K98" s="6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L98" s="6" t="inlineStr"/>
       <c r="M98" s="6" t="inlineStr">
         <is>
@@ -10993,9 +11209,17 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="I99" s="6" t="inlineStr"/>
+      <c r="I99" s="6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="J99" s="6" t="inlineStr"/>
-      <c r="K99" s="6" t="inlineStr"/>
+      <c r="K99" s="6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L99" s="6" t="inlineStr"/>
       <c r="M99" s="6" t="inlineStr">
         <is>
@@ -11090,9 +11314,17 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="I100" s="6" t="inlineStr"/>
+      <c r="I100" s="6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="J100" s="6" t="inlineStr"/>
-      <c r="K100" s="6" t="inlineStr"/>
+      <c r="K100" s="6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L100" s="6" t="inlineStr"/>
       <c r="M100" s="6" t="inlineStr">
         <is>
@@ -11187,9 +11419,17 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="I101" s="6" t="inlineStr"/>
+      <c r="I101" s="6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="J101" s="6" t="inlineStr"/>
-      <c r="K101" s="6" t="inlineStr"/>
+      <c r="K101" s="6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L101" s="6" t="inlineStr"/>
       <c r="M101" s="6" t="inlineStr">
         <is>
@@ -11284,9 +11524,17 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="I102" s="6" t="inlineStr"/>
+      <c r="I102" s="6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="J102" s="6" t="inlineStr"/>
-      <c r="K102" s="6" t="inlineStr"/>
+      <c r="K102" s="6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L102" s="6" t="inlineStr"/>
       <c r="M102" s="6" t="inlineStr">
         <is>
@@ -11381,9 +11629,17 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="I103" s="6" t="inlineStr"/>
+      <c r="I103" s="6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="J103" s="6" t="inlineStr"/>
-      <c r="K103" s="6" t="inlineStr"/>
+      <c r="K103" s="6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L103" s="6" t="inlineStr"/>
       <c r="M103" s="6" t="inlineStr">
         <is>
@@ -11478,9 +11734,17 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="I104" s="6" t="inlineStr"/>
+      <c r="I104" s="6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="J104" s="6" t="inlineStr"/>
-      <c r="K104" s="6" t="inlineStr"/>
+      <c r="K104" s="6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L104" s="6" t="inlineStr"/>
       <c r="M104" s="6" t="inlineStr">
         <is>
@@ -11575,9 +11839,17 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="I105" s="6" t="inlineStr"/>
+      <c r="I105" s="6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="J105" s="6" t="inlineStr"/>
-      <c r="K105" s="6" t="inlineStr"/>
+      <c r="K105" s="6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L105" s="6" t="inlineStr"/>
       <c r="M105" s="6" t="inlineStr">
         <is>
@@ -11672,9 +11944,17 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="I106" s="6" t="inlineStr"/>
+      <c r="I106" s="6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="J106" s="6" t="inlineStr"/>
-      <c r="K106" s="6" t="inlineStr"/>
+      <c r="K106" s="6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L106" s="6" t="inlineStr"/>
       <c r="M106" s="6" t="inlineStr">
         <is>
@@ -11769,9 +12049,17 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="I107" s="6" t="inlineStr"/>
+      <c r="I107" s="6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="J107" s="6" t="inlineStr"/>
-      <c r="K107" s="6" t="inlineStr"/>
+      <c r="K107" s="6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L107" s="6" t="inlineStr"/>
       <c r="M107" s="6" t="inlineStr">
         <is>
@@ -11866,9 +12154,17 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="I108" s="6" t="inlineStr"/>
+      <c r="I108" s="6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="J108" s="6" t="inlineStr"/>
-      <c r="K108" s="6" t="inlineStr"/>
+      <c r="K108" s="6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L108" s="6" t="inlineStr"/>
       <c r="M108" s="6" t="inlineStr">
         <is>
@@ -11963,9 +12259,17 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="I109" s="6" t="inlineStr"/>
+      <c r="I109" s="6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="J109" s="6" t="inlineStr"/>
-      <c r="K109" s="6" t="inlineStr"/>
+      <c r="K109" s="6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L109" s="6" t="inlineStr"/>
       <c r="M109" s="6" t="inlineStr">
         <is>
@@ -12060,9 +12364,17 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="I110" s="6" t="inlineStr"/>
+      <c r="I110" s="6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="J110" s="6" t="inlineStr"/>
-      <c r="K110" s="6" t="inlineStr"/>
+      <c r="K110" s="6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L110" s="6" t="inlineStr"/>
       <c r="M110" s="6" t="inlineStr">
         <is>
@@ -12157,9 +12469,17 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="I111" s="6" t="inlineStr"/>
+      <c r="I111" s="6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="J111" s="6" t="inlineStr"/>
-      <c r="K111" s="6" t="inlineStr"/>
+      <c r="K111" s="6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L111" s="6" t="inlineStr"/>
       <c r="M111" s="6" t="inlineStr">
         <is>
@@ -12254,9 +12574,17 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="I112" s="6" t="inlineStr"/>
+      <c r="I112" s="6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="J112" s="6" t="inlineStr"/>
-      <c r="K112" s="6" t="inlineStr"/>
+      <c r="K112" s="6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L112" s="6" t="inlineStr"/>
       <c r="M112" s="6" t="inlineStr">
         <is>

</xml_diff>